<commit_message>
feat(legacy-services): renombrar Total, ordenamiento por columnas y edición/eliminación de registros
</commit_message>
<xml_diff>
--- a/public/templates/plantilla_servicios_legacy.xlsx
+++ b/public/templates/plantilla_servicios_legacy.xlsx
@@ -483,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q1000"/>
+  <dimension ref="A1:P1000"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -501,8 +501,7 @@
     <col width="22" customWidth="1" min="13" max="13"/>
     <col width="14" customWidth="1" min="14" max="14"/>
     <col width="32" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="40" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="38" customHeight="1">
@@ -573,17 +572,12 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>Subtotal</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Observaciones internas</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Total</t>
         </is>
       </c>
     </row>
@@ -649,10 +643,7 @@
         <v>30000</v>
       </c>
       <c r="O2" s="2" t="inlineStr"/>
-      <c r="P2" s="3" t="n">
-        <v>35700</v>
-      </c>
-      <c r="Q2" s="4" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>← FILA EJEMPLO (bórrela antes de cargar)</t>
         </is>
@@ -660,3995 +651,2997 @@
     </row>
     <row r="3">
       <c r="N3" s="5" t="n"/>
-      <c r="P3" s="5" t="n"/>
     </row>
     <row r="4">
       <c r="N4" s="5" t="n"/>
-      <c r="P4" s="5" t="n"/>
     </row>
     <row r="5">
       <c r="N5" s="5" t="n"/>
-      <c r="P5" s="5" t="n"/>
     </row>
     <row r="6">
       <c r="N6" s="5" t="n"/>
-      <c r="P6" s="5" t="n"/>
     </row>
     <row r="7">
       <c r="N7" s="5" t="n"/>
-      <c r="P7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="N8" s="5" t="n"/>
-      <c r="P8" s="5" t="n"/>
     </row>
     <row r="9">
       <c r="N9" s="5" t="n"/>
-      <c r="P9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="N10" s="5" t="n"/>
-      <c r="P10" s="5" t="n"/>
     </row>
     <row r="11">
       <c r="N11" s="5" t="n"/>
-      <c r="P11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="N12" s="5" t="n"/>
-      <c r="P12" s="5" t="n"/>
     </row>
     <row r="13">
       <c r="N13" s="5" t="n"/>
-      <c r="P13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="N14" s="5" t="n"/>
-      <c r="P14" s="5" t="n"/>
     </row>
     <row r="15">
       <c r="N15" s="5" t="n"/>
-      <c r="P15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="N16" s="5" t="n"/>
-      <c r="P16" s="5" t="n"/>
     </row>
     <row r="17">
       <c r="N17" s="5" t="n"/>
-      <c r="P17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="N18" s="5" t="n"/>
-      <c r="P18" s="5" t="n"/>
     </row>
     <row r="19">
       <c r="N19" s="5" t="n"/>
-      <c r="P19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="N20" s="5" t="n"/>
-      <c r="P20" s="5" t="n"/>
     </row>
     <row r="21">
       <c r="N21" s="5" t="n"/>
-      <c r="P21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="N22" s="5" t="n"/>
-      <c r="P22" s="5" t="n"/>
     </row>
     <row r="23">
       <c r="N23" s="5" t="n"/>
-      <c r="P23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="N24" s="5" t="n"/>
-      <c r="P24" s="5" t="n"/>
     </row>
     <row r="25">
       <c r="N25" s="5" t="n"/>
-      <c r="P25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="N26" s="5" t="n"/>
-      <c r="P26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="N27" s="5" t="n"/>
-      <c r="P27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="N28" s="5" t="n"/>
-      <c r="P28" s="5" t="n"/>
     </row>
     <row r="29">
       <c r="N29" s="5" t="n"/>
-      <c r="P29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="N30" s="5" t="n"/>
-      <c r="P30" s="5" t="n"/>
     </row>
     <row r="31">
       <c r="N31" s="5" t="n"/>
-      <c r="P31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="N32" s="5" t="n"/>
-      <c r="P32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="N33" s="5" t="n"/>
-      <c r="P33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="N34" s="5" t="n"/>
-      <c r="P34" s="5" t="n"/>
     </row>
     <row r="35">
       <c r="N35" s="5" t="n"/>
-      <c r="P35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="N36" s="5" t="n"/>
-      <c r="P36" s="5" t="n"/>
     </row>
     <row r="37">
       <c r="N37" s="5" t="n"/>
-      <c r="P37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="N38" s="5" t="n"/>
-      <c r="P38" s="5" t="n"/>
     </row>
     <row r="39">
       <c r="N39" s="5" t="n"/>
-      <c r="P39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="N40" s="5" t="n"/>
-      <c r="P40" s="5" t="n"/>
     </row>
     <row r="41">
       <c r="N41" s="5" t="n"/>
-      <c r="P41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="N42" s="5" t="n"/>
-      <c r="P42" s="5" t="n"/>
     </row>
     <row r="43">
       <c r="N43" s="5" t="n"/>
-      <c r="P43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="N44" s="5" t="n"/>
-      <c r="P44" s="5" t="n"/>
     </row>
     <row r="45">
       <c r="N45" s="5" t="n"/>
-      <c r="P45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="N46" s="5" t="n"/>
-      <c r="P46" s="5" t="n"/>
     </row>
     <row r="47">
       <c r="N47" s="5" t="n"/>
-      <c r="P47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="N48" s="5" t="n"/>
-      <c r="P48" s="5" t="n"/>
     </row>
     <row r="49">
       <c r="N49" s="5" t="n"/>
-      <c r="P49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="N50" s="5" t="n"/>
-      <c r="P50" s="5" t="n"/>
     </row>
     <row r="51">
       <c r="N51" s="5" t="n"/>
-      <c r="P51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="N52" s="5" t="n"/>
-      <c r="P52" s="5" t="n"/>
     </row>
     <row r="53">
       <c r="N53" s="5" t="n"/>
-      <c r="P53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="N54" s="5" t="n"/>
-      <c r="P54" s="5" t="n"/>
     </row>
     <row r="55">
       <c r="N55" s="5" t="n"/>
-      <c r="P55" s="5" t="n"/>
     </row>
     <row r="56">
       <c r="N56" s="5" t="n"/>
-      <c r="P56" s="5" t="n"/>
     </row>
     <row r="57">
       <c r="N57" s="5" t="n"/>
-      <c r="P57" s="5" t="n"/>
     </row>
     <row r="58">
       <c r="N58" s="5" t="n"/>
-      <c r="P58" s="5" t="n"/>
     </row>
     <row r="59">
       <c r="N59" s="5" t="n"/>
-      <c r="P59" s="5" t="n"/>
     </row>
     <row r="60">
       <c r="N60" s="5" t="n"/>
-      <c r="P60" s="5" t="n"/>
     </row>
     <row r="61">
       <c r="N61" s="5" t="n"/>
-      <c r="P61" s="5" t="n"/>
     </row>
     <row r="62">
       <c r="N62" s="5" t="n"/>
-      <c r="P62" s="5" t="n"/>
     </row>
     <row r="63">
       <c r="N63" s="5" t="n"/>
-      <c r="P63" s="5" t="n"/>
     </row>
     <row r="64">
       <c r="N64" s="5" t="n"/>
-      <c r="P64" s="5" t="n"/>
     </row>
     <row r="65">
       <c r="N65" s="5" t="n"/>
-      <c r="P65" s="5" t="n"/>
     </row>
     <row r="66">
       <c r="N66" s="5" t="n"/>
-      <c r="P66" s="5" t="n"/>
     </row>
     <row r="67">
       <c r="N67" s="5" t="n"/>
-      <c r="P67" s="5" t="n"/>
     </row>
     <row r="68">
       <c r="N68" s="5" t="n"/>
-      <c r="P68" s="5" t="n"/>
     </row>
     <row r="69">
       <c r="N69" s="5" t="n"/>
-      <c r="P69" s="5" t="n"/>
     </row>
     <row r="70">
       <c r="N70" s="5" t="n"/>
-      <c r="P70" s="5" t="n"/>
     </row>
     <row r="71">
       <c r="N71" s="5" t="n"/>
-      <c r="P71" s="5" t="n"/>
     </row>
     <row r="72">
       <c r="N72" s="5" t="n"/>
-      <c r="P72" s="5" t="n"/>
     </row>
     <row r="73">
       <c r="N73" s="5" t="n"/>
-      <c r="P73" s="5" t="n"/>
     </row>
     <row r="74">
       <c r="N74" s="5" t="n"/>
-      <c r="P74" s="5" t="n"/>
     </row>
     <row r="75">
       <c r="N75" s="5" t="n"/>
-      <c r="P75" s="5" t="n"/>
     </row>
     <row r="76">
       <c r="N76" s="5" t="n"/>
-      <c r="P76" s="5" t="n"/>
     </row>
     <row r="77">
       <c r="N77" s="5" t="n"/>
-      <c r="P77" s="5" t="n"/>
     </row>
     <row r="78">
       <c r="N78" s="5" t="n"/>
-      <c r="P78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="N79" s="5" t="n"/>
-      <c r="P79" s="5" t="n"/>
     </row>
     <row r="80">
       <c r="N80" s="5" t="n"/>
-      <c r="P80" s="5" t="n"/>
     </row>
     <row r="81">
       <c r="N81" s="5" t="n"/>
-      <c r="P81" s="5" t="n"/>
     </row>
     <row r="82">
       <c r="N82" s="5" t="n"/>
-      <c r="P82" s="5" t="n"/>
     </row>
     <row r="83">
       <c r="N83" s="5" t="n"/>
-      <c r="P83" s="5" t="n"/>
     </row>
     <row r="84">
       <c r="N84" s="5" t="n"/>
-      <c r="P84" s="5" t="n"/>
     </row>
     <row r="85">
       <c r="N85" s="5" t="n"/>
-      <c r="P85" s="5" t="n"/>
     </row>
     <row r="86">
       <c r="N86" s="5" t="n"/>
-      <c r="P86" s="5" t="n"/>
     </row>
     <row r="87">
       <c r="N87" s="5" t="n"/>
-      <c r="P87" s="5" t="n"/>
     </row>
     <row r="88">
       <c r="N88" s="5" t="n"/>
-      <c r="P88" s="5" t="n"/>
     </row>
     <row r="89">
       <c r="N89" s="5" t="n"/>
-      <c r="P89" s="5" t="n"/>
     </row>
     <row r="90">
       <c r="N90" s="5" t="n"/>
-      <c r="P90" s="5" t="n"/>
     </row>
     <row r="91">
       <c r="N91" s="5" t="n"/>
-      <c r="P91" s="5" t="n"/>
     </row>
     <row r="92">
       <c r="N92" s="5" t="n"/>
-      <c r="P92" s="5" t="n"/>
     </row>
     <row r="93">
       <c r="N93" s="5" t="n"/>
-      <c r="P93" s="5" t="n"/>
     </row>
     <row r="94">
       <c r="N94" s="5" t="n"/>
-      <c r="P94" s="5" t="n"/>
     </row>
     <row r="95">
       <c r="N95" s="5" t="n"/>
-      <c r="P95" s="5" t="n"/>
     </row>
     <row r="96">
       <c r="N96" s="5" t="n"/>
-      <c r="P96" s="5" t="n"/>
     </row>
     <row r="97">
       <c r="N97" s="5" t="n"/>
-      <c r="P97" s="5" t="n"/>
     </row>
     <row r="98">
       <c r="N98" s="5" t="n"/>
-      <c r="P98" s="5" t="n"/>
     </row>
     <row r="99">
       <c r="N99" s="5" t="n"/>
-      <c r="P99" s="5" t="n"/>
     </row>
     <row r="100">
       <c r="N100" s="5" t="n"/>
-      <c r="P100" s="5" t="n"/>
     </row>
     <row r="101">
       <c r="N101" s="5" t="n"/>
-      <c r="P101" s="5" t="n"/>
     </row>
     <row r="102">
       <c r="N102" s="5" t="n"/>
-      <c r="P102" s="5" t="n"/>
     </row>
     <row r="103">
       <c r="N103" s="5" t="n"/>
-      <c r="P103" s="5" t="n"/>
     </row>
     <row r="104">
       <c r="N104" s="5" t="n"/>
-      <c r="P104" s="5" t="n"/>
     </row>
     <row r="105">
       <c r="N105" s="5" t="n"/>
-      <c r="P105" s="5" t="n"/>
     </row>
     <row r="106">
       <c r="N106" s="5" t="n"/>
-      <c r="P106" s="5" t="n"/>
     </row>
     <row r="107">
       <c r="N107" s="5" t="n"/>
-      <c r="P107" s="5" t="n"/>
     </row>
     <row r="108">
       <c r="N108" s="5" t="n"/>
-      <c r="P108" s="5" t="n"/>
     </row>
     <row r="109">
       <c r="N109" s="5" t="n"/>
-      <c r="P109" s="5" t="n"/>
     </row>
     <row r="110">
       <c r="N110" s="5" t="n"/>
-      <c r="P110" s="5" t="n"/>
     </row>
     <row r="111">
       <c r="N111" s="5" t="n"/>
-      <c r="P111" s="5" t="n"/>
     </row>
     <row r="112">
       <c r="N112" s="5" t="n"/>
-      <c r="P112" s="5" t="n"/>
     </row>
     <row r="113">
       <c r="N113" s="5" t="n"/>
-      <c r="P113" s="5" t="n"/>
     </row>
     <row r="114">
       <c r="N114" s="5" t="n"/>
-      <c r="P114" s="5" t="n"/>
     </row>
     <row r="115">
       <c r="N115" s="5" t="n"/>
-      <c r="P115" s="5" t="n"/>
     </row>
     <row r="116">
       <c r="N116" s="5" t="n"/>
-      <c r="P116" s="5" t="n"/>
     </row>
     <row r="117">
       <c r="N117" s="5" t="n"/>
-      <c r="P117" s="5" t="n"/>
     </row>
     <row r="118">
       <c r="N118" s="5" t="n"/>
-      <c r="P118" s="5" t="n"/>
     </row>
     <row r="119">
       <c r="N119" s="5" t="n"/>
-      <c r="P119" s="5" t="n"/>
     </row>
     <row r="120">
       <c r="N120" s="5" t="n"/>
-      <c r="P120" s="5" t="n"/>
     </row>
     <row r="121">
       <c r="N121" s="5" t="n"/>
-      <c r="P121" s="5" t="n"/>
     </row>
     <row r="122">
       <c r="N122" s="5" t="n"/>
-      <c r="P122" s="5" t="n"/>
     </row>
     <row r="123">
       <c r="N123" s="5" t="n"/>
-      <c r="P123" s="5" t="n"/>
     </row>
     <row r="124">
       <c r="N124" s="5" t="n"/>
-      <c r="P124" s="5" t="n"/>
     </row>
     <row r="125">
       <c r="N125" s="5" t="n"/>
-      <c r="P125" s="5" t="n"/>
     </row>
     <row r="126">
       <c r="N126" s="5" t="n"/>
-      <c r="P126" s="5" t="n"/>
     </row>
     <row r="127">
       <c r="N127" s="5" t="n"/>
-      <c r="P127" s="5" t="n"/>
     </row>
     <row r="128">
       <c r="N128" s="5" t="n"/>
-      <c r="P128" s="5" t="n"/>
     </row>
     <row r="129">
       <c r="N129" s="5" t="n"/>
-      <c r="P129" s="5" t="n"/>
     </row>
     <row r="130">
       <c r="N130" s="5" t="n"/>
-      <c r="P130" s="5" t="n"/>
     </row>
     <row r="131">
       <c r="N131" s="5" t="n"/>
-      <c r="P131" s="5" t="n"/>
     </row>
     <row r="132">
       <c r="N132" s="5" t="n"/>
-      <c r="P132" s="5" t="n"/>
     </row>
     <row r="133">
       <c r="N133" s="5" t="n"/>
-      <c r="P133" s="5" t="n"/>
     </row>
     <row r="134">
       <c r="N134" s="5" t="n"/>
-      <c r="P134" s="5" t="n"/>
     </row>
     <row r="135">
       <c r="N135" s="5" t="n"/>
-      <c r="P135" s="5" t="n"/>
     </row>
     <row r="136">
       <c r="N136" s="5" t="n"/>
-      <c r="P136" s="5" t="n"/>
     </row>
     <row r="137">
       <c r="N137" s="5" t="n"/>
-      <c r="P137" s="5" t="n"/>
     </row>
     <row r="138">
       <c r="N138" s="5" t="n"/>
-      <c r="P138" s="5" t="n"/>
     </row>
     <row r="139">
       <c r="N139" s="5" t="n"/>
-      <c r="P139" s="5" t="n"/>
     </row>
     <row r="140">
       <c r="N140" s="5" t="n"/>
-      <c r="P140" s="5" t="n"/>
     </row>
     <row r="141">
       <c r="N141" s="5" t="n"/>
-      <c r="P141" s="5" t="n"/>
     </row>
     <row r="142">
       <c r="N142" s="5" t="n"/>
-      <c r="P142" s="5" t="n"/>
     </row>
     <row r="143">
       <c r="N143" s="5" t="n"/>
-      <c r="P143" s="5" t="n"/>
     </row>
     <row r="144">
       <c r="N144" s="5" t="n"/>
-      <c r="P144" s="5" t="n"/>
     </row>
     <row r="145">
       <c r="N145" s="5" t="n"/>
-      <c r="P145" s="5" t="n"/>
     </row>
     <row r="146">
       <c r="N146" s="5" t="n"/>
-      <c r="P146" s="5" t="n"/>
     </row>
     <row r="147">
       <c r="N147" s="5" t="n"/>
-      <c r="P147" s="5" t="n"/>
     </row>
     <row r="148">
       <c r="N148" s="5" t="n"/>
-      <c r="P148" s="5" t="n"/>
     </row>
     <row r="149">
       <c r="N149" s="5" t="n"/>
-      <c r="P149" s="5" t="n"/>
     </row>
     <row r="150">
       <c r="N150" s="5" t="n"/>
-      <c r="P150" s="5" t="n"/>
     </row>
     <row r="151">
       <c r="N151" s="5" t="n"/>
-      <c r="P151" s="5" t="n"/>
     </row>
     <row r="152">
       <c r="N152" s="5" t="n"/>
-      <c r="P152" s="5" t="n"/>
     </row>
     <row r="153">
       <c r="N153" s="5" t="n"/>
-      <c r="P153" s="5" t="n"/>
     </row>
     <row r="154">
       <c r="N154" s="5" t="n"/>
-      <c r="P154" s="5" t="n"/>
     </row>
     <row r="155">
       <c r="N155" s="5" t="n"/>
-      <c r="P155" s="5" t="n"/>
     </row>
     <row r="156">
       <c r="N156" s="5" t="n"/>
-      <c r="P156" s="5" t="n"/>
     </row>
     <row r="157">
       <c r="N157" s="5" t="n"/>
-      <c r="P157" s="5" t="n"/>
     </row>
     <row r="158">
       <c r="N158" s="5" t="n"/>
-      <c r="P158" s="5" t="n"/>
     </row>
     <row r="159">
       <c r="N159" s="5" t="n"/>
-      <c r="P159" s="5" t="n"/>
     </row>
     <row r="160">
       <c r="N160" s="5" t="n"/>
-      <c r="P160" s="5" t="n"/>
     </row>
     <row r="161">
       <c r="N161" s="5" t="n"/>
-      <c r="P161" s="5" t="n"/>
     </row>
     <row r="162">
       <c r="N162" s="5" t="n"/>
-      <c r="P162" s="5" t="n"/>
     </row>
     <row r="163">
       <c r="N163" s="5" t="n"/>
-      <c r="P163" s="5" t="n"/>
     </row>
     <row r="164">
       <c r="N164" s="5" t="n"/>
-      <c r="P164" s="5" t="n"/>
     </row>
     <row r="165">
       <c r="N165" s="5" t="n"/>
-      <c r="P165" s="5" t="n"/>
     </row>
     <row r="166">
       <c r="N166" s="5" t="n"/>
-      <c r="P166" s="5" t="n"/>
     </row>
     <row r="167">
       <c r="N167" s="5" t="n"/>
-      <c r="P167" s="5" t="n"/>
     </row>
     <row r="168">
       <c r="N168" s="5" t="n"/>
-      <c r="P168" s="5" t="n"/>
     </row>
     <row r="169">
       <c r="N169" s="5" t="n"/>
-      <c r="P169" s="5" t="n"/>
     </row>
     <row r="170">
       <c r="N170" s="5" t="n"/>
-      <c r="P170" s="5" t="n"/>
     </row>
     <row r="171">
       <c r="N171" s="5" t="n"/>
-      <c r="P171" s="5" t="n"/>
     </row>
     <row r="172">
       <c r="N172" s="5" t="n"/>
-      <c r="P172" s="5" t="n"/>
     </row>
     <row r="173">
       <c r="N173" s="5" t="n"/>
-      <c r="P173" s="5" t="n"/>
     </row>
     <row r="174">
       <c r="N174" s="5" t="n"/>
-      <c r="P174" s="5" t="n"/>
     </row>
     <row r="175">
       <c r="N175" s="5" t="n"/>
-      <c r="P175" s="5" t="n"/>
     </row>
     <row r="176">
       <c r="N176" s="5" t="n"/>
-      <c r="P176" s="5" t="n"/>
     </row>
     <row r="177">
       <c r="N177" s="5" t="n"/>
-      <c r="P177" s="5" t="n"/>
     </row>
     <row r="178">
       <c r="N178" s="5" t="n"/>
-      <c r="P178" s="5" t="n"/>
     </row>
     <row r="179">
       <c r="N179" s="5" t="n"/>
-      <c r="P179" s="5" t="n"/>
     </row>
     <row r="180">
       <c r="N180" s="5" t="n"/>
-      <c r="P180" s="5" t="n"/>
     </row>
     <row r="181">
       <c r="N181" s="5" t="n"/>
-      <c r="P181" s="5" t="n"/>
     </row>
     <row r="182">
       <c r="N182" s="5" t="n"/>
-      <c r="P182" s="5" t="n"/>
     </row>
     <row r="183">
       <c r="N183" s="5" t="n"/>
-      <c r="P183" s="5" t="n"/>
     </row>
     <row r="184">
       <c r="N184" s="5" t="n"/>
-      <c r="P184" s="5" t="n"/>
     </row>
     <row r="185">
       <c r="N185" s="5" t="n"/>
-      <c r="P185" s="5" t="n"/>
     </row>
     <row r="186">
       <c r="N186" s="5" t="n"/>
-      <c r="P186" s="5" t="n"/>
     </row>
     <row r="187">
       <c r="N187" s="5" t="n"/>
-      <c r="P187" s="5" t="n"/>
     </row>
     <row r="188">
       <c r="N188" s="5" t="n"/>
-      <c r="P188" s="5" t="n"/>
     </row>
     <row r="189">
       <c r="N189" s="5" t="n"/>
-      <c r="P189" s="5" t="n"/>
     </row>
     <row r="190">
       <c r="N190" s="5" t="n"/>
-      <c r="P190" s="5" t="n"/>
     </row>
     <row r="191">
       <c r="N191" s="5" t="n"/>
-      <c r="P191" s="5" t="n"/>
     </row>
     <row r="192">
       <c r="N192" s="5" t="n"/>
-      <c r="P192" s="5" t="n"/>
     </row>
     <row r="193">
       <c r="N193" s="5" t="n"/>
-      <c r="P193" s="5" t="n"/>
     </row>
     <row r="194">
       <c r="N194" s="5" t="n"/>
-      <c r="P194" s="5" t="n"/>
     </row>
     <row r="195">
       <c r="N195" s="5" t="n"/>
-      <c r="P195" s="5" t="n"/>
     </row>
     <row r="196">
       <c r="N196" s="5" t="n"/>
-      <c r="P196" s="5" t="n"/>
     </row>
     <row r="197">
       <c r="N197" s="5" t="n"/>
-      <c r="P197" s="5" t="n"/>
     </row>
     <row r="198">
       <c r="N198" s="5" t="n"/>
-      <c r="P198" s="5" t="n"/>
     </row>
     <row r="199">
       <c r="N199" s="5" t="n"/>
-      <c r="P199" s="5" t="n"/>
     </row>
     <row r="200">
       <c r="N200" s="5" t="n"/>
-      <c r="P200" s="5" t="n"/>
     </row>
     <row r="201">
       <c r="N201" s="5" t="n"/>
-      <c r="P201" s="5" t="n"/>
     </row>
     <row r="202">
       <c r="N202" s="5" t="n"/>
-      <c r="P202" s="5" t="n"/>
     </row>
     <row r="203">
       <c r="N203" s="5" t="n"/>
-      <c r="P203" s="5" t="n"/>
     </row>
     <row r="204">
       <c r="N204" s="5" t="n"/>
-      <c r="P204" s="5" t="n"/>
     </row>
     <row r="205">
       <c r="N205" s="5" t="n"/>
-      <c r="P205" s="5" t="n"/>
     </row>
     <row r="206">
       <c r="N206" s="5" t="n"/>
-      <c r="P206" s="5" t="n"/>
     </row>
     <row r="207">
       <c r="N207" s="5" t="n"/>
-      <c r="P207" s="5" t="n"/>
     </row>
     <row r="208">
       <c r="N208" s="5" t="n"/>
-      <c r="P208" s="5" t="n"/>
     </row>
     <row r="209">
       <c r="N209" s="5" t="n"/>
-      <c r="P209" s="5" t="n"/>
     </row>
     <row r="210">
       <c r="N210" s="5" t="n"/>
-      <c r="P210" s="5" t="n"/>
     </row>
     <row r="211">
       <c r="N211" s="5" t="n"/>
-      <c r="P211" s="5" t="n"/>
     </row>
     <row r="212">
       <c r="N212" s="5" t="n"/>
-      <c r="P212" s="5" t="n"/>
     </row>
     <row r="213">
       <c r="N213" s="5" t="n"/>
-      <c r="P213" s="5" t="n"/>
     </row>
     <row r="214">
       <c r="N214" s="5" t="n"/>
-      <c r="P214" s="5" t="n"/>
     </row>
     <row r="215">
       <c r="N215" s="5" t="n"/>
-      <c r="P215" s="5" t="n"/>
     </row>
     <row r="216">
       <c r="N216" s="5" t="n"/>
-      <c r="P216" s="5" t="n"/>
     </row>
     <row r="217">
       <c r="N217" s="5" t="n"/>
-      <c r="P217" s="5" t="n"/>
     </row>
     <row r="218">
       <c r="N218" s="5" t="n"/>
-      <c r="P218" s="5" t="n"/>
     </row>
     <row r="219">
       <c r="N219" s="5" t="n"/>
-      <c r="P219" s="5" t="n"/>
     </row>
     <row r="220">
       <c r="N220" s="5" t="n"/>
-      <c r="P220" s="5" t="n"/>
     </row>
     <row r="221">
       <c r="N221" s="5" t="n"/>
-      <c r="P221" s="5" t="n"/>
     </row>
     <row r="222">
       <c r="N222" s="5" t="n"/>
-      <c r="P222" s="5" t="n"/>
     </row>
     <row r="223">
       <c r="N223" s="5" t="n"/>
-      <c r="P223" s="5" t="n"/>
     </row>
     <row r="224">
       <c r="N224" s="5" t="n"/>
-      <c r="P224" s="5" t="n"/>
     </row>
     <row r="225">
       <c r="N225" s="5" t="n"/>
-      <c r="P225" s="5" t="n"/>
     </row>
     <row r="226">
       <c r="N226" s="5" t="n"/>
-      <c r="P226" s="5" t="n"/>
     </row>
     <row r="227">
       <c r="N227" s="5" t="n"/>
-      <c r="P227" s="5" t="n"/>
     </row>
     <row r="228">
       <c r="N228" s="5" t="n"/>
-      <c r="P228" s="5" t="n"/>
     </row>
     <row r="229">
       <c r="N229" s="5" t="n"/>
-      <c r="P229" s="5" t="n"/>
     </row>
     <row r="230">
       <c r="N230" s="5" t="n"/>
-      <c r="P230" s="5" t="n"/>
     </row>
     <row r="231">
       <c r="N231" s="5" t="n"/>
-      <c r="P231" s="5" t="n"/>
     </row>
     <row r="232">
       <c r="N232" s="5" t="n"/>
-      <c r="P232" s="5" t="n"/>
     </row>
     <row r="233">
       <c r="N233" s="5" t="n"/>
-      <c r="P233" s="5" t="n"/>
     </row>
     <row r="234">
       <c r="N234" s="5" t="n"/>
-      <c r="P234" s="5" t="n"/>
     </row>
     <row r="235">
       <c r="N235" s="5" t="n"/>
-      <c r="P235" s="5" t="n"/>
     </row>
     <row r="236">
       <c r="N236" s="5" t="n"/>
-      <c r="P236" s="5" t="n"/>
     </row>
     <row r="237">
       <c r="N237" s="5" t="n"/>
-      <c r="P237" s="5" t="n"/>
     </row>
     <row r="238">
       <c r="N238" s="5" t="n"/>
-      <c r="P238" s="5" t="n"/>
     </row>
     <row r="239">
       <c r="N239" s="5" t="n"/>
-      <c r="P239" s="5" t="n"/>
     </row>
     <row r="240">
       <c r="N240" s="5" t="n"/>
-      <c r="P240" s="5" t="n"/>
     </row>
     <row r="241">
       <c r="N241" s="5" t="n"/>
-      <c r="P241" s="5" t="n"/>
     </row>
     <row r="242">
       <c r="N242" s="5" t="n"/>
-      <c r="P242" s="5" t="n"/>
     </row>
     <row r="243">
       <c r="N243" s="5" t="n"/>
-      <c r="P243" s="5" t="n"/>
     </row>
     <row r="244">
       <c r="N244" s="5" t="n"/>
-      <c r="P244" s="5" t="n"/>
     </row>
     <row r="245">
       <c r="N245" s="5" t="n"/>
-      <c r="P245" s="5" t="n"/>
     </row>
     <row r="246">
       <c r="N246" s="5" t="n"/>
-      <c r="P246" s="5" t="n"/>
     </row>
     <row r="247">
       <c r="N247" s="5" t="n"/>
-      <c r="P247" s="5" t="n"/>
     </row>
     <row r="248">
       <c r="N248" s="5" t="n"/>
-      <c r="P248" s="5" t="n"/>
     </row>
     <row r="249">
       <c r="N249" s="5" t="n"/>
-      <c r="P249" s="5" t="n"/>
     </row>
     <row r="250">
       <c r="N250" s="5" t="n"/>
-      <c r="P250" s="5" t="n"/>
     </row>
     <row r="251">
       <c r="N251" s="5" t="n"/>
-      <c r="P251" s="5" t="n"/>
     </row>
     <row r="252">
       <c r="N252" s="5" t="n"/>
-      <c r="P252" s="5" t="n"/>
     </row>
     <row r="253">
       <c r="N253" s="5" t="n"/>
-      <c r="P253" s="5" t="n"/>
     </row>
     <row r="254">
       <c r="N254" s="5" t="n"/>
-      <c r="P254" s="5" t="n"/>
     </row>
     <row r="255">
       <c r="N255" s="5" t="n"/>
-      <c r="P255" s="5" t="n"/>
     </row>
     <row r="256">
       <c r="N256" s="5" t="n"/>
-      <c r="P256" s="5" t="n"/>
     </row>
     <row r="257">
       <c r="N257" s="5" t="n"/>
-      <c r="P257" s="5" t="n"/>
     </row>
     <row r="258">
       <c r="N258" s="5" t="n"/>
-      <c r="P258" s="5" t="n"/>
     </row>
     <row r="259">
       <c r="N259" s="5" t="n"/>
-      <c r="P259" s="5" t="n"/>
     </row>
     <row r="260">
       <c r="N260" s="5" t="n"/>
-      <c r="P260" s="5" t="n"/>
     </row>
     <row r="261">
       <c r="N261" s="5" t="n"/>
-      <c r="P261" s="5" t="n"/>
     </row>
     <row r="262">
       <c r="N262" s="5" t="n"/>
-      <c r="P262" s="5" t="n"/>
     </row>
     <row r="263">
       <c r="N263" s="5" t="n"/>
-      <c r="P263" s="5" t="n"/>
     </row>
     <row r="264">
       <c r="N264" s="5" t="n"/>
-      <c r="P264" s="5" t="n"/>
     </row>
     <row r="265">
       <c r="N265" s="5" t="n"/>
-      <c r="P265" s="5" t="n"/>
     </row>
     <row r="266">
       <c r="N266" s="5" t="n"/>
-      <c r="P266" s="5" t="n"/>
     </row>
     <row r="267">
       <c r="N267" s="5" t="n"/>
-      <c r="P267" s="5" t="n"/>
     </row>
     <row r="268">
       <c r="N268" s="5" t="n"/>
-      <c r="P268" s="5" t="n"/>
     </row>
     <row r="269">
       <c r="N269" s="5" t="n"/>
-      <c r="P269" s="5" t="n"/>
     </row>
     <row r="270">
       <c r="N270" s="5" t="n"/>
-      <c r="P270" s="5" t="n"/>
     </row>
     <row r="271">
       <c r="N271" s="5" t="n"/>
-      <c r="P271" s="5" t="n"/>
     </row>
     <row r="272">
       <c r="N272" s="5" t="n"/>
-      <c r="P272" s="5" t="n"/>
     </row>
     <row r="273">
       <c r="N273" s="5" t="n"/>
-      <c r="P273" s="5" t="n"/>
     </row>
     <row r="274">
       <c r="N274" s="5" t="n"/>
-      <c r="P274" s="5" t="n"/>
     </row>
     <row r="275">
       <c r="N275" s="5" t="n"/>
-      <c r="P275" s="5" t="n"/>
     </row>
     <row r="276">
       <c r="N276" s="5" t="n"/>
-      <c r="P276" s="5" t="n"/>
     </row>
     <row r="277">
       <c r="N277" s="5" t="n"/>
-      <c r="P277" s="5" t="n"/>
     </row>
     <row r="278">
       <c r="N278" s="5" t="n"/>
-      <c r="P278" s="5" t="n"/>
     </row>
     <row r="279">
       <c r="N279" s="5" t="n"/>
-      <c r="P279" s="5" t="n"/>
     </row>
     <row r="280">
       <c r="N280" s="5" t="n"/>
-      <c r="P280" s="5" t="n"/>
     </row>
     <row r="281">
       <c r="N281" s="5" t="n"/>
-      <c r="P281" s="5" t="n"/>
     </row>
     <row r="282">
       <c r="N282" s="5" t="n"/>
-      <c r="P282" s="5" t="n"/>
     </row>
     <row r="283">
       <c r="N283" s="5" t="n"/>
-      <c r="P283" s="5" t="n"/>
     </row>
     <row r="284">
       <c r="N284" s="5" t="n"/>
-      <c r="P284" s="5" t="n"/>
     </row>
     <row r="285">
       <c r="N285" s="5" t="n"/>
-      <c r="P285" s="5" t="n"/>
     </row>
     <row r="286">
       <c r="N286" s="5" t="n"/>
-      <c r="P286" s="5" t="n"/>
     </row>
     <row r="287">
       <c r="N287" s="5" t="n"/>
-      <c r="P287" s="5" t="n"/>
     </row>
     <row r="288">
       <c r="N288" s="5" t="n"/>
-      <c r="P288" s="5" t="n"/>
     </row>
     <row r="289">
       <c r="N289" s="5" t="n"/>
-      <c r="P289" s="5" t="n"/>
     </row>
     <row r="290">
       <c r="N290" s="5" t="n"/>
-      <c r="P290" s="5" t="n"/>
     </row>
     <row r="291">
       <c r="N291" s="5" t="n"/>
-      <c r="P291" s="5" t="n"/>
     </row>
     <row r="292">
       <c r="N292" s="5" t="n"/>
-      <c r="P292" s="5" t="n"/>
     </row>
     <row r="293">
       <c r="N293" s="5" t="n"/>
-      <c r="P293" s="5" t="n"/>
     </row>
     <row r="294">
       <c r="N294" s="5" t="n"/>
-      <c r="P294" s="5" t="n"/>
     </row>
     <row r="295">
       <c r="N295" s="5" t="n"/>
-      <c r="P295" s="5" t="n"/>
     </row>
     <row r="296">
       <c r="N296" s="5" t="n"/>
-      <c r="P296" s="5" t="n"/>
     </row>
     <row r="297">
       <c r="N297" s="5" t="n"/>
-      <c r="P297" s="5" t="n"/>
     </row>
     <row r="298">
       <c r="N298" s="5" t="n"/>
-      <c r="P298" s="5" t="n"/>
     </row>
     <row r="299">
       <c r="N299" s="5" t="n"/>
-      <c r="P299" s="5" t="n"/>
     </row>
     <row r="300">
       <c r="N300" s="5" t="n"/>
-      <c r="P300" s="5" t="n"/>
     </row>
     <row r="301">
       <c r="N301" s="5" t="n"/>
-      <c r="P301" s="5" t="n"/>
     </row>
     <row r="302">
       <c r="N302" s="5" t="n"/>
-      <c r="P302" s="5" t="n"/>
     </row>
     <row r="303">
       <c r="N303" s="5" t="n"/>
-      <c r="P303" s="5" t="n"/>
     </row>
     <row r="304">
       <c r="N304" s="5" t="n"/>
-      <c r="P304" s="5" t="n"/>
     </row>
     <row r="305">
       <c r="N305" s="5" t="n"/>
-      <c r="P305" s="5" t="n"/>
     </row>
     <row r="306">
       <c r="N306" s="5" t="n"/>
-      <c r="P306" s="5" t="n"/>
     </row>
     <row r="307">
       <c r="N307" s="5" t="n"/>
-      <c r="P307" s="5" t="n"/>
     </row>
     <row r="308">
       <c r="N308" s="5" t="n"/>
-      <c r="P308" s="5" t="n"/>
     </row>
     <row r="309">
       <c r="N309" s="5" t="n"/>
-      <c r="P309" s="5" t="n"/>
     </row>
     <row r="310">
       <c r="N310" s="5" t="n"/>
-      <c r="P310" s="5" t="n"/>
     </row>
     <row r="311">
       <c r="N311" s="5" t="n"/>
-      <c r="P311" s="5" t="n"/>
     </row>
     <row r="312">
       <c r="N312" s="5" t="n"/>
-      <c r="P312" s="5" t="n"/>
     </row>
     <row r="313">
       <c r="N313" s="5" t="n"/>
-      <c r="P313" s="5" t="n"/>
     </row>
     <row r="314">
       <c r="N314" s="5" t="n"/>
-      <c r="P314" s="5" t="n"/>
     </row>
     <row r="315">
       <c r="N315" s="5" t="n"/>
-      <c r="P315" s="5" t="n"/>
     </row>
     <row r="316">
       <c r="N316" s="5" t="n"/>
-      <c r="P316" s="5" t="n"/>
     </row>
     <row r="317">
       <c r="N317" s="5" t="n"/>
-      <c r="P317" s="5" t="n"/>
     </row>
     <row r="318">
       <c r="N318" s="5" t="n"/>
-      <c r="P318" s="5" t="n"/>
     </row>
     <row r="319">
       <c r="N319" s="5" t="n"/>
-      <c r="P319" s="5" t="n"/>
     </row>
     <row r="320">
       <c r="N320" s="5" t="n"/>
-      <c r="P320" s="5" t="n"/>
     </row>
     <row r="321">
       <c r="N321" s="5" t="n"/>
-      <c r="P321" s="5" t="n"/>
     </row>
     <row r="322">
       <c r="N322" s="5" t="n"/>
-      <c r="P322" s="5" t="n"/>
     </row>
     <row r="323">
       <c r="N323" s="5" t="n"/>
-      <c r="P323" s="5" t="n"/>
     </row>
     <row r="324">
       <c r="N324" s="5" t="n"/>
-      <c r="P324" s="5" t="n"/>
     </row>
     <row r="325">
       <c r="N325" s="5" t="n"/>
-      <c r="P325" s="5" t="n"/>
     </row>
     <row r="326">
       <c r="N326" s="5" t="n"/>
-      <c r="P326" s="5" t="n"/>
     </row>
     <row r="327">
       <c r="N327" s="5" t="n"/>
-      <c r="P327" s="5" t="n"/>
     </row>
     <row r="328">
       <c r="N328" s="5" t="n"/>
-      <c r="P328" s="5" t="n"/>
     </row>
     <row r="329">
       <c r="N329" s="5" t="n"/>
-      <c r="P329" s="5" t="n"/>
     </row>
     <row r="330">
       <c r="N330" s="5" t="n"/>
-      <c r="P330" s="5" t="n"/>
     </row>
     <row r="331">
       <c r="N331" s="5" t="n"/>
-      <c r="P331" s="5" t="n"/>
     </row>
     <row r="332">
       <c r="N332" s="5" t="n"/>
-      <c r="P332" s="5" t="n"/>
     </row>
     <row r="333">
       <c r="N333" s="5" t="n"/>
-      <c r="P333" s="5" t="n"/>
     </row>
     <row r="334">
       <c r="N334" s="5" t="n"/>
-      <c r="P334" s="5" t="n"/>
     </row>
     <row r="335">
       <c r="N335" s="5" t="n"/>
-      <c r="P335" s="5" t="n"/>
     </row>
     <row r="336">
       <c r="N336" s="5" t="n"/>
-      <c r="P336" s="5" t="n"/>
     </row>
     <row r="337">
       <c r="N337" s="5" t="n"/>
-      <c r="P337" s="5" t="n"/>
     </row>
     <row r="338">
       <c r="N338" s="5" t="n"/>
-      <c r="P338" s="5" t="n"/>
     </row>
     <row r="339">
       <c r="N339" s="5" t="n"/>
-      <c r="P339" s="5" t="n"/>
     </row>
     <row r="340">
       <c r="N340" s="5" t="n"/>
-      <c r="P340" s="5" t="n"/>
     </row>
     <row r="341">
       <c r="N341" s="5" t="n"/>
-      <c r="P341" s="5" t="n"/>
     </row>
     <row r="342">
       <c r="N342" s="5" t="n"/>
-      <c r="P342" s="5" t="n"/>
     </row>
     <row r="343">
       <c r="N343" s="5" t="n"/>
-      <c r="P343" s="5" t="n"/>
     </row>
     <row r="344">
       <c r="N344" s="5" t="n"/>
-      <c r="P344" s="5" t="n"/>
     </row>
     <row r="345">
       <c r="N345" s="5" t="n"/>
-      <c r="P345" s="5" t="n"/>
     </row>
     <row r="346">
       <c r="N346" s="5" t="n"/>
-      <c r="P346" s="5" t="n"/>
     </row>
     <row r="347">
       <c r="N347" s="5" t="n"/>
-      <c r="P347" s="5" t="n"/>
     </row>
     <row r="348">
       <c r="N348" s="5" t="n"/>
-      <c r="P348" s="5" t="n"/>
     </row>
     <row r="349">
       <c r="N349" s="5" t="n"/>
-      <c r="P349" s="5" t="n"/>
     </row>
     <row r="350">
       <c r="N350" s="5" t="n"/>
-      <c r="P350" s="5" t="n"/>
     </row>
     <row r="351">
       <c r="N351" s="5" t="n"/>
-      <c r="P351" s="5" t="n"/>
     </row>
     <row r="352">
       <c r="N352" s="5" t="n"/>
-      <c r="P352" s="5" t="n"/>
     </row>
     <row r="353">
       <c r="N353" s="5" t="n"/>
-      <c r="P353" s="5" t="n"/>
     </row>
     <row r="354">
       <c r="N354" s="5" t="n"/>
-      <c r="P354" s="5" t="n"/>
     </row>
     <row r="355">
       <c r="N355" s="5" t="n"/>
-      <c r="P355" s="5" t="n"/>
     </row>
     <row r="356">
       <c r="N356" s="5" t="n"/>
-      <c r="P356" s="5" t="n"/>
     </row>
     <row r="357">
       <c r="N357" s="5" t="n"/>
-      <c r="P357" s="5" t="n"/>
     </row>
     <row r="358">
       <c r="N358" s="5" t="n"/>
-      <c r="P358" s="5" t="n"/>
     </row>
     <row r="359">
       <c r="N359" s="5" t="n"/>
-      <c r="P359" s="5" t="n"/>
     </row>
     <row r="360">
       <c r="N360" s="5" t="n"/>
-      <c r="P360" s="5" t="n"/>
     </row>
     <row r="361">
       <c r="N361" s="5" t="n"/>
-      <c r="P361" s="5" t="n"/>
     </row>
     <row r="362">
       <c r="N362" s="5" t="n"/>
-      <c r="P362" s="5" t="n"/>
     </row>
     <row r="363">
       <c r="N363" s="5" t="n"/>
-      <c r="P363" s="5" t="n"/>
     </row>
     <row r="364">
       <c r="N364" s="5" t="n"/>
-      <c r="P364" s="5" t="n"/>
     </row>
     <row r="365">
       <c r="N365" s="5" t="n"/>
-      <c r="P365" s="5" t="n"/>
     </row>
     <row r="366">
       <c r="N366" s="5" t="n"/>
-      <c r="P366" s="5" t="n"/>
     </row>
     <row r="367">
       <c r="N367" s="5" t="n"/>
-      <c r="P367" s="5" t="n"/>
     </row>
     <row r="368">
       <c r="N368" s="5" t="n"/>
-      <c r="P368" s="5" t="n"/>
     </row>
     <row r="369">
       <c r="N369" s="5" t="n"/>
-      <c r="P369" s="5" t="n"/>
     </row>
     <row r="370">
       <c r="N370" s="5" t="n"/>
-      <c r="P370" s="5" t="n"/>
     </row>
     <row r="371">
       <c r="N371" s="5" t="n"/>
-      <c r="P371" s="5" t="n"/>
     </row>
     <row r="372">
       <c r="N372" s="5" t="n"/>
-      <c r="P372" s="5" t="n"/>
     </row>
     <row r="373">
       <c r="N373" s="5" t="n"/>
-      <c r="P373" s="5" t="n"/>
     </row>
     <row r="374">
       <c r="N374" s="5" t="n"/>
-      <c r="P374" s="5" t="n"/>
     </row>
     <row r="375">
       <c r="N375" s="5" t="n"/>
-      <c r="P375" s="5" t="n"/>
     </row>
     <row r="376">
       <c r="N376" s="5" t="n"/>
-      <c r="P376" s="5" t="n"/>
     </row>
     <row r="377">
       <c r="N377" s="5" t="n"/>
-      <c r="P377" s="5" t="n"/>
     </row>
     <row r="378">
       <c r="N378" s="5" t="n"/>
-      <c r="P378" s="5" t="n"/>
     </row>
     <row r="379">
       <c r="N379" s="5" t="n"/>
-      <c r="P379" s="5" t="n"/>
     </row>
     <row r="380">
       <c r="N380" s="5" t="n"/>
-      <c r="P380" s="5" t="n"/>
     </row>
     <row r="381">
       <c r="N381" s="5" t="n"/>
-      <c r="P381" s="5" t="n"/>
     </row>
     <row r="382">
       <c r="N382" s="5" t="n"/>
-      <c r="P382" s="5" t="n"/>
     </row>
     <row r="383">
       <c r="N383" s="5" t="n"/>
-      <c r="P383" s="5" t="n"/>
     </row>
     <row r="384">
       <c r="N384" s="5" t="n"/>
-      <c r="P384" s="5" t="n"/>
     </row>
     <row r="385">
       <c r="N385" s="5" t="n"/>
-      <c r="P385" s="5" t="n"/>
     </row>
     <row r="386">
       <c r="N386" s="5" t="n"/>
-      <c r="P386" s="5" t="n"/>
     </row>
     <row r="387">
       <c r="N387" s="5" t="n"/>
-      <c r="P387" s="5" t="n"/>
     </row>
     <row r="388">
       <c r="N388" s="5" t="n"/>
-      <c r="P388" s="5" t="n"/>
     </row>
     <row r="389">
       <c r="N389" s="5" t="n"/>
-      <c r="P389" s="5" t="n"/>
     </row>
     <row r="390">
       <c r="N390" s="5" t="n"/>
-      <c r="P390" s="5" t="n"/>
     </row>
     <row r="391">
       <c r="N391" s="5" t="n"/>
-      <c r="P391" s="5" t="n"/>
     </row>
     <row r="392">
       <c r="N392" s="5" t="n"/>
-      <c r="P392" s="5" t="n"/>
     </row>
     <row r="393">
       <c r="N393" s="5" t="n"/>
-      <c r="P393" s="5" t="n"/>
     </row>
     <row r="394">
       <c r="N394" s="5" t="n"/>
-      <c r="P394" s="5" t="n"/>
     </row>
     <row r="395">
       <c r="N395" s="5" t="n"/>
-      <c r="P395" s="5" t="n"/>
     </row>
     <row r="396">
       <c r="N396" s="5" t="n"/>
-      <c r="P396" s="5" t="n"/>
     </row>
     <row r="397">
       <c r="N397" s="5" t="n"/>
-      <c r="P397" s="5" t="n"/>
     </row>
     <row r="398">
       <c r="N398" s="5" t="n"/>
-      <c r="P398" s="5" t="n"/>
     </row>
     <row r="399">
       <c r="N399" s="5" t="n"/>
-      <c r="P399" s="5" t="n"/>
     </row>
     <row r="400">
       <c r="N400" s="5" t="n"/>
-      <c r="P400" s="5" t="n"/>
     </row>
     <row r="401">
       <c r="N401" s="5" t="n"/>
-      <c r="P401" s="5" t="n"/>
     </row>
     <row r="402">
       <c r="N402" s="5" t="n"/>
-      <c r="P402" s="5" t="n"/>
     </row>
     <row r="403">
       <c r="N403" s="5" t="n"/>
-      <c r="P403" s="5" t="n"/>
     </row>
     <row r="404">
       <c r="N404" s="5" t="n"/>
-      <c r="P404" s="5" t="n"/>
     </row>
     <row r="405">
       <c r="N405" s="5" t="n"/>
-      <c r="P405" s="5" t="n"/>
     </row>
     <row r="406">
       <c r="N406" s="5" t="n"/>
-      <c r="P406" s="5" t="n"/>
     </row>
     <row r="407">
       <c r="N407" s="5" t="n"/>
-      <c r="P407" s="5" t="n"/>
     </row>
     <row r="408">
       <c r="N408" s="5" t="n"/>
-      <c r="P408" s="5" t="n"/>
     </row>
     <row r="409">
       <c r="N409" s="5" t="n"/>
-      <c r="P409" s="5" t="n"/>
     </row>
     <row r="410">
       <c r="N410" s="5" t="n"/>
-      <c r="P410" s="5" t="n"/>
     </row>
     <row r="411">
       <c r="N411" s="5" t="n"/>
-      <c r="P411" s="5" t="n"/>
     </row>
     <row r="412">
       <c r="N412" s="5" t="n"/>
-      <c r="P412" s="5" t="n"/>
     </row>
     <row r="413">
       <c r="N413" s="5" t="n"/>
-      <c r="P413" s="5" t="n"/>
     </row>
     <row r="414">
       <c r="N414" s="5" t="n"/>
-      <c r="P414" s="5" t="n"/>
     </row>
     <row r="415">
       <c r="N415" s="5" t="n"/>
-      <c r="P415" s="5" t="n"/>
     </row>
     <row r="416">
       <c r="N416" s="5" t="n"/>
-      <c r="P416" s="5" t="n"/>
     </row>
     <row r="417">
       <c r="N417" s="5" t="n"/>
-      <c r="P417" s="5" t="n"/>
     </row>
     <row r="418">
       <c r="N418" s="5" t="n"/>
-      <c r="P418" s="5" t="n"/>
     </row>
     <row r="419">
       <c r="N419" s="5" t="n"/>
-      <c r="P419" s="5" t="n"/>
     </row>
     <row r="420">
       <c r="N420" s="5" t="n"/>
-      <c r="P420" s="5" t="n"/>
     </row>
     <row r="421">
       <c r="N421" s="5" t="n"/>
-      <c r="P421" s="5" t="n"/>
     </row>
     <row r="422">
       <c r="N422" s="5" t="n"/>
-      <c r="P422" s="5" t="n"/>
     </row>
     <row r="423">
       <c r="N423" s="5" t="n"/>
-      <c r="P423" s="5" t="n"/>
     </row>
     <row r="424">
       <c r="N424" s="5" t="n"/>
-      <c r="P424" s="5" t="n"/>
     </row>
     <row r="425">
       <c r="N425" s="5" t="n"/>
-      <c r="P425" s="5" t="n"/>
     </row>
     <row r="426">
       <c r="N426" s="5" t="n"/>
-      <c r="P426" s="5" t="n"/>
     </row>
     <row r="427">
       <c r="N427" s="5" t="n"/>
-      <c r="P427" s="5" t="n"/>
     </row>
     <row r="428">
       <c r="N428" s="5" t="n"/>
-      <c r="P428" s="5" t="n"/>
     </row>
     <row r="429">
       <c r="N429" s="5" t="n"/>
-      <c r="P429" s="5" t="n"/>
     </row>
     <row r="430">
       <c r="N430" s="5" t="n"/>
-      <c r="P430" s="5" t="n"/>
     </row>
     <row r="431">
       <c r="N431" s="5" t="n"/>
-      <c r="P431" s="5" t="n"/>
     </row>
     <row r="432">
       <c r="N432" s="5" t="n"/>
-      <c r="P432" s="5" t="n"/>
     </row>
     <row r="433">
       <c r="N433" s="5" t="n"/>
-      <c r="P433" s="5" t="n"/>
     </row>
     <row r="434">
       <c r="N434" s="5" t="n"/>
-      <c r="P434" s="5" t="n"/>
     </row>
     <row r="435">
       <c r="N435" s="5" t="n"/>
-      <c r="P435" s="5" t="n"/>
     </row>
     <row r="436">
       <c r="N436" s="5" t="n"/>
-      <c r="P436" s="5" t="n"/>
     </row>
     <row r="437">
       <c r="N437" s="5" t="n"/>
-      <c r="P437" s="5" t="n"/>
     </row>
     <row r="438">
       <c r="N438" s="5" t="n"/>
-      <c r="P438" s="5" t="n"/>
     </row>
     <row r="439">
       <c r="N439" s="5" t="n"/>
-      <c r="P439" s="5" t="n"/>
     </row>
     <row r="440">
       <c r="N440" s="5" t="n"/>
-      <c r="P440" s="5" t="n"/>
     </row>
     <row r="441">
       <c r="N441" s="5" t="n"/>
-      <c r="P441" s="5" t="n"/>
     </row>
     <row r="442">
       <c r="N442" s="5" t="n"/>
-      <c r="P442" s="5" t="n"/>
     </row>
     <row r="443">
       <c r="N443" s="5" t="n"/>
-      <c r="P443" s="5" t="n"/>
     </row>
     <row r="444">
       <c r="N444" s="5" t="n"/>
-      <c r="P444" s="5" t="n"/>
     </row>
     <row r="445">
       <c r="N445" s="5" t="n"/>
-      <c r="P445" s="5" t="n"/>
     </row>
     <row r="446">
       <c r="N446" s="5" t="n"/>
-      <c r="P446" s="5" t="n"/>
     </row>
     <row r="447">
       <c r="N447" s="5" t="n"/>
-      <c r="P447" s="5" t="n"/>
     </row>
     <row r="448">
       <c r="N448" s="5" t="n"/>
-      <c r="P448" s="5" t="n"/>
     </row>
     <row r="449">
       <c r="N449" s="5" t="n"/>
-      <c r="P449" s="5" t="n"/>
     </row>
     <row r="450">
       <c r="N450" s="5" t="n"/>
-      <c r="P450" s="5" t="n"/>
     </row>
     <row r="451">
       <c r="N451" s="5" t="n"/>
-      <c r="P451" s="5" t="n"/>
     </row>
     <row r="452">
       <c r="N452" s="5" t="n"/>
-      <c r="P452" s="5" t="n"/>
     </row>
     <row r="453">
       <c r="N453" s="5" t="n"/>
-      <c r="P453" s="5" t="n"/>
     </row>
     <row r="454">
       <c r="N454" s="5" t="n"/>
-      <c r="P454" s="5" t="n"/>
     </row>
     <row r="455">
       <c r="N455" s="5" t="n"/>
-      <c r="P455" s="5" t="n"/>
     </row>
     <row r="456">
       <c r="N456" s="5" t="n"/>
-      <c r="P456" s="5" t="n"/>
     </row>
     <row r="457">
       <c r="N457" s="5" t="n"/>
-      <c r="P457" s="5" t="n"/>
     </row>
     <row r="458">
       <c r="N458" s="5" t="n"/>
-      <c r="P458" s="5" t="n"/>
     </row>
     <row r="459">
       <c r="N459" s="5" t="n"/>
-      <c r="P459" s="5" t="n"/>
     </row>
     <row r="460">
       <c r="N460" s="5" t="n"/>
-      <c r="P460" s="5" t="n"/>
     </row>
     <row r="461">
       <c r="N461" s="5" t="n"/>
-      <c r="P461" s="5" t="n"/>
     </row>
     <row r="462">
       <c r="N462" s="5" t="n"/>
-      <c r="P462" s="5" t="n"/>
     </row>
     <row r="463">
       <c r="N463" s="5" t="n"/>
-      <c r="P463" s="5" t="n"/>
     </row>
     <row r="464">
       <c r="N464" s="5" t="n"/>
-      <c r="P464" s="5" t="n"/>
     </row>
     <row r="465">
       <c r="N465" s="5" t="n"/>
-      <c r="P465" s="5" t="n"/>
     </row>
     <row r="466">
       <c r="N466" s="5" t="n"/>
-      <c r="P466" s="5" t="n"/>
     </row>
     <row r="467">
       <c r="N467" s="5" t="n"/>
-      <c r="P467" s="5" t="n"/>
     </row>
     <row r="468">
       <c r="N468" s="5" t="n"/>
-      <c r="P468" s="5" t="n"/>
     </row>
     <row r="469">
       <c r="N469" s="5" t="n"/>
-      <c r="P469" s="5" t="n"/>
     </row>
     <row r="470">
       <c r="N470" s="5" t="n"/>
-      <c r="P470" s="5" t="n"/>
     </row>
     <row r="471">
       <c r="N471" s="5" t="n"/>
-      <c r="P471" s="5" t="n"/>
     </row>
     <row r="472">
       <c r="N472" s="5" t="n"/>
-      <c r="P472" s="5" t="n"/>
     </row>
     <row r="473">
       <c r="N473" s="5" t="n"/>
-      <c r="P473" s="5" t="n"/>
     </row>
     <row r="474">
       <c r="N474" s="5" t="n"/>
-      <c r="P474" s="5" t="n"/>
     </row>
     <row r="475">
       <c r="N475" s="5" t="n"/>
-      <c r="P475" s="5" t="n"/>
     </row>
     <row r="476">
       <c r="N476" s="5" t="n"/>
-      <c r="P476" s="5" t="n"/>
     </row>
     <row r="477">
       <c r="N477" s="5" t="n"/>
-      <c r="P477" s="5" t="n"/>
     </row>
     <row r="478">
       <c r="N478" s="5" t="n"/>
-      <c r="P478" s="5" t="n"/>
     </row>
     <row r="479">
       <c r="N479" s="5" t="n"/>
-      <c r="P479" s="5" t="n"/>
     </row>
     <row r="480">
       <c r="N480" s="5" t="n"/>
-      <c r="P480" s="5" t="n"/>
     </row>
     <row r="481">
       <c r="N481" s="5" t="n"/>
-      <c r="P481" s="5" t="n"/>
     </row>
     <row r="482">
       <c r="N482" s="5" t="n"/>
-      <c r="P482" s="5" t="n"/>
     </row>
     <row r="483">
       <c r="N483" s="5" t="n"/>
-      <c r="P483" s="5" t="n"/>
     </row>
     <row r="484">
       <c r="N484" s="5" t="n"/>
-      <c r="P484" s="5" t="n"/>
     </row>
     <row r="485">
       <c r="N485" s="5" t="n"/>
-      <c r="P485" s="5" t="n"/>
     </row>
     <row r="486">
       <c r="N486" s="5" t="n"/>
-      <c r="P486" s="5" t="n"/>
     </row>
     <row r="487">
       <c r="N487" s="5" t="n"/>
-      <c r="P487" s="5" t="n"/>
     </row>
     <row r="488">
       <c r="N488" s="5" t="n"/>
-      <c r="P488" s="5" t="n"/>
     </row>
     <row r="489">
       <c r="N489" s="5" t="n"/>
-      <c r="P489" s="5" t="n"/>
     </row>
     <row r="490">
       <c r="N490" s="5" t="n"/>
-      <c r="P490" s="5" t="n"/>
     </row>
     <row r="491">
       <c r="N491" s="5" t="n"/>
-      <c r="P491" s="5" t="n"/>
     </row>
     <row r="492">
       <c r="N492" s="5" t="n"/>
-      <c r="P492" s="5" t="n"/>
     </row>
     <row r="493">
       <c r="N493" s="5" t="n"/>
-      <c r="P493" s="5" t="n"/>
     </row>
     <row r="494">
       <c r="N494" s="5" t="n"/>
-      <c r="P494" s="5" t="n"/>
     </row>
     <row r="495">
       <c r="N495" s="5" t="n"/>
-      <c r="P495" s="5" t="n"/>
     </row>
     <row r="496">
       <c r="N496" s="5" t="n"/>
-      <c r="P496" s="5" t="n"/>
     </row>
     <row r="497">
       <c r="N497" s="5" t="n"/>
-      <c r="P497" s="5" t="n"/>
     </row>
     <row r="498">
       <c r="N498" s="5" t="n"/>
-      <c r="P498" s="5" t="n"/>
     </row>
     <row r="499">
       <c r="N499" s="5" t="n"/>
-      <c r="P499" s="5" t="n"/>
     </row>
     <row r="500">
       <c r="N500" s="5" t="n"/>
-      <c r="P500" s="5" t="n"/>
     </row>
     <row r="501">
       <c r="N501" s="5" t="n"/>
-      <c r="P501" s="5" t="n"/>
     </row>
     <row r="502">
       <c r="N502" s="5" t="n"/>
-      <c r="P502" s="5" t="n"/>
     </row>
     <row r="503">
       <c r="N503" s="5" t="n"/>
-      <c r="P503" s="5" t="n"/>
     </row>
     <row r="504">
       <c r="N504" s="5" t="n"/>
-      <c r="P504" s="5" t="n"/>
     </row>
     <row r="505">
       <c r="N505" s="5" t="n"/>
-      <c r="P505" s="5" t="n"/>
     </row>
     <row r="506">
       <c r="N506" s="5" t="n"/>
-      <c r="P506" s="5" t="n"/>
     </row>
     <row r="507">
       <c r="N507" s="5" t="n"/>
-      <c r="P507" s="5" t="n"/>
     </row>
     <row r="508">
       <c r="N508" s="5" t="n"/>
-      <c r="P508" s="5" t="n"/>
     </row>
     <row r="509">
       <c r="N509" s="5" t="n"/>
-      <c r="P509" s="5" t="n"/>
     </row>
     <row r="510">
       <c r="N510" s="5" t="n"/>
-      <c r="P510" s="5" t="n"/>
     </row>
     <row r="511">
       <c r="N511" s="5" t="n"/>
-      <c r="P511" s="5" t="n"/>
     </row>
     <row r="512">
       <c r="N512" s="5" t="n"/>
-      <c r="P512" s="5" t="n"/>
     </row>
     <row r="513">
       <c r="N513" s="5" t="n"/>
-      <c r="P513" s="5" t="n"/>
     </row>
     <row r="514">
       <c r="N514" s="5" t="n"/>
-      <c r="P514" s="5" t="n"/>
     </row>
     <row r="515">
       <c r="N515" s="5" t="n"/>
-      <c r="P515" s="5" t="n"/>
     </row>
     <row r="516">
       <c r="N516" s="5" t="n"/>
-      <c r="P516" s="5" t="n"/>
     </row>
     <row r="517">
       <c r="N517" s="5" t="n"/>
-      <c r="P517" s="5" t="n"/>
     </row>
     <row r="518">
       <c r="N518" s="5" t="n"/>
-      <c r="P518" s="5" t="n"/>
     </row>
     <row r="519">
       <c r="N519" s="5" t="n"/>
-      <c r="P519" s="5" t="n"/>
     </row>
     <row r="520">
       <c r="N520" s="5" t="n"/>
-      <c r="P520" s="5" t="n"/>
     </row>
     <row r="521">
       <c r="N521" s="5" t="n"/>
-      <c r="P521" s="5" t="n"/>
     </row>
     <row r="522">
       <c r="N522" s="5" t="n"/>
-      <c r="P522" s="5" t="n"/>
     </row>
     <row r="523">
       <c r="N523" s="5" t="n"/>
-      <c r="P523" s="5" t="n"/>
     </row>
     <row r="524">
       <c r="N524" s="5" t="n"/>
-      <c r="P524" s="5" t="n"/>
     </row>
     <row r="525">
       <c r="N525" s="5" t="n"/>
-      <c r="P525" s="5" t="n"/>
     </row>
     <row r="526">
       <c r="N526" s="5" t="n"/>
-      <c r="P526" s="5" t="n"/>
     </row>
     <row r="527">
       <c r="N527" s="5" t="n"/>
-      <c r="P527" s="5" t="n"/>
     </row>
     <row r="528">
       <c r="N528" s="5" t="n"/>
-      <c r="P528" s="5" t="n"/>
     </row>
     <row r="529">
       <c r="N529" s="5" t="n"/>
-      <c r="P529" s="5" t="n"/>
     </row>
     <row r="530">
       <c r="N530" s="5" t="n"/>
-      <c r="P530" s="5" t="n"/>
     </row>
     <row r="531">
       <c r="N531" s="5" t="n"/>
-      <c r="P531" s="5" t="n"/>
     </row>
     <row r="532">
       <c r="N532" s="5" t="n"/>
-      <c r="P532" s="5" t="n"/>
     </row>
     <row r="533">
       <c r="N533" s="5" t="n"/>
-      <c r="P533" s="5" t="n"/>
     </row>
     <row r="534">
       <c r="N534" s="5" t="n"/>
-      <c r="P534" s="5" t="n"/>
     </row>
     <row r="535">
       <c r="N535" s="5" t="n"/>
-      <c r="P535" s="5" t="n"/>
     </row>
     <row r="536">
       <c r="N536" s="5" t="n"/>
-      <c r="P536" s="5" t="n"/>
     </row>
     <row r="537">
       <c r="N537" s="5" t="n"/>
-      <c r="P537" s="5" t="n"/>
     </row>
     <row r="538">
       <c r="N538" s="5" t="n"/>
-      <c r="P538" s="5" t="n"/>
     </row>
     <row r="539">
       <c r="N539" s="5" t="n"/>
-      <c r="P539" s="5" t="n"/>
     </row>
     <row r="540">
       <c r="N540" s="5" t="n"/>
-      <c r="P540" s="5" t="n"/>
     </row>
     <row r="541">
       <c r="N541" s="5" t="n"/>
-      <c r="P541" s="5" t="n"/>
     </row>
     <row r="542">
       <c r="N542" s="5" t="n"/>
-      <c r="P542" s="5" t="n"/>
     </row>
     <row r="543">
       <c r="N543" s="5" t="n"/>
-      <c r="P543" s="5" t="n"/>
     </row>
     <row r="544">
       <c r="N544" s="5" t="n"/>
-      <c r="P544" s="5" t="n"/>
     </row>
     <row r="545">
       <c r="N545" s="5" t="n"/>
-      <c r="P545" s="5" t="n"/>
     </row>
     <row r="546">
       <c r="N546" s="5" t="n"/>
-      <c r="P546" s="5" t="n"/>
     </row>
     <row r="547">
       <c r="N547" s="5" t="n"/>
-      <c r="P547" s="5" t="n"/>
     </row>
     <row r="548">
       <c r="N548" s="5" t="n"/>
-      <c r="P548" s="5" t="n"/>
     </row>
     <row r="549">
       <c r="N549" s="5" t="n"/>
-      <c r="P549" s="5" t="n"/>
     </row>
     <row r="550">
       <c r="N550" s="5" t="n"/>
-      <c r="P550" s="5" t="n"/>
     </row>
     <row r="551">
       <c r="N551" s="5" t="n"/>
-      <c r="P551" s="5" t="n"/>
     </row>
     <row r="552">
       <c r="N552" s="5" t="n"/>
-      <c r="P552" s="5" t="n"/>
     </row>
     <row r="553">
       <c r="N553" s="5" t="n"/>
-      <c r="P553" s="5" t="n"/>
     </row>
     <row r="554">
       <c r="N554" s="5" t="n"/>
-      <c r="P554" s="5" t="n"/>
     </row>
     <row r="555">
       <c r="N555" s="5" t="n"/>
-      <c r="P555" s="5" t="n"/>
     </row>
     <row r="556">
       <c r="N556" s="5" t="n"/>
-      <c r="P556" s="5" t="n"/>
     </row>
     <row r="557">
       <c r="N557" s="5" t="n"/>
-      <c r="P557" s="5" t="n"/>
     </row>
     <row r="558">
       <c r="N558" s="5" t="n"/>
-      <c r="P558" s="5" t="n"/>
     </row>
     <row r="559">
       <c r="N559" s="5" t="n"/>
-      <c r="P559" s="5" t="n"/>
     </row>
     <row r="560">
       <c r="N560" s="5" t="n"/>
-      <c r="P560" s="5" t="n"/>
     </row>
     <row r="561">
       <c r="N561" s="5" t="n"/>
-      <c r="P561" s="5" t="n"/>
     </row>
     <row r="562">
       <c r="N562" s="5" t="n"/>
-      <c r="P562" s="5" t="n"/>
     </row>
     <row r="563">
       <c r="N563" s="5" t="n"/>
-      <c r="P563" s="5" t="n"/>
     </row>
     <row r="564">
       <c r="N564" s="5" t="n"/>
-      <c r="P564" s="5" t="n"/>
     </row>
     <row r="565">
       <c r="N565" s="5" t="n"/>
-      <c r="P565" s="5" t="n"/>
     </row>
     <row r="566">
       <c r="N566" s="5" t="n"/>
-      <c r="P566" s="5" t="n"/>
     </row>
     <row r="567">
       <c r="N567" s="5" t="n"/>
-      <c r="P567" s="5" t="n"/>
     </row>
     <row r="568">
       <c r="N568" s="5" t="n"/>
-      <c r="P568" s="5" t="n"/>
     </row>
     <row r="569">
       <c r="N569" s="5" t="n"/>
-      <c r="P569" s="5" t="n"/>
     </row>
     <row r="570">
       <c r="N570" s="5" t="n"/>
-      <c r="P570" s="5" t="n"/>
     </row>
     <row r="571">
       <c r="N571" s="5" t="n"/>
-      <c r="P571" s="5" t="n"/>
     </row>
     <row r="572">
       <c r="N572" s="5" t="n"/>
-      <c r="P572" s="5" t="n"/>
     </row>
     <row r="573">
       <c r="N573" s="5" t="n"/>
-      <c r="P573" s="5" t="n"/>
     </row>
     <row r="574">
       <c r="N574" s="5" t="n"/>
-      <c r="P574" s="5" t="n"/>
     </row>
     <row r="575">
       <c r="N575" s="5" t="n"/>
-      <c r="P575" s="5" t="n"/>
     </row>
     <row r="576">
       <c r="N576" s="5" t="n"/>
-      <c r="P576" s="5" t="n"/>
     </row>
     <row r="577">
       <c r="N577" s="5" t="n"/>
-      <c r="P577" s="5" t="n"/>
     </row>
     <row r="578">
       <c r="N578" s="5" t="n"/>
-      <c r="P578" s="5" t="n"/>
     </row>
     <row r="579">
       <c r="N579" s="5" t="n"/>
-      <c r="P579" s="5" t="n"/>
     </row>
     <row r="580">
       <c r="N580" s="5" t="n"/>
-      <c r="P580" s="5" t="n"/>
     </row>
     <row r="581">
       <c r="N581" s="5" t="n"/>
-      <c r="P581" s="5" t="n"/>
     </row>
     <row r="582">
       <c r="N582" s="5" t="n"/>
-      <c r="P582" s="5" t="n"/>
     </row>
     <row r="583">
       <c r="N583" s="5" t="n"/>
-      <c r="P583" s="5" t="n"/>
     </row>
     <row r="584">
       <c r="N584" s="5" t="n"/>
-      <c r="P584" s="5" t="n"/>
     </row>
     <row r="585">
       <c r="N585" s="5" t="n"/>
-      <c r="P585" s="5" t="n"/>
     </row>
     <row r="586">
       <c r="N586" s="5" t="n"/>
-      <c r="P586" s="5" t="n"/>
     </row>
     <row r="587">
       <c r="N587" s="5" t="n"/>
-      <c r="P587" s="5" t="n"/>
     </row>
     <row r="588">
       <c r="N588" s="5" t="n"/>
-      <c r="P588" s="5" t="n"/>
     </row>
     <row r="589">
       <c r="N589" s="5" t="n"/>
-      <c r="P589" s="5" t="n"/>
     </row>
     <row r="590">
       <c r="N590" s="5" t="n"/>
-      <c r="P590" s="5" t="n"/>
     </row>
     <row r="591">
       <c r="N591" s="5" t="n"/>
-      <c r="P591" s="5" t="n"/>
     </row>
     <row r="592">
       <c r="N592" s="5" t="n"/>
-      <c r="P592" s="5" t="n"/>
     </row>
     <row r="593">
       <c r="N593" s="5" t="n"/>
-      <c r="P593" s="5" t="n"/>
     </row>
     <row r="594">
       <c r="N594" s="5" t="n"/>
-      <c r="P594" s="5" t="n"/>
     </row>
     <row r="595">
       <c r="N595" s="5" t="n"/>
-      <c r="P595" s="5" t="n"/>
     </row>
     <row r="596">
       <c r="N596" s="5" t="n"/>
-      <c r="P596" s="5" t="n"/>
     </row>
     <row r="597">
       <c r="N597" s="5" t="n"/>
-      <c r="P597" s="5" t="n"/>
     </row>
     <row r="598">
       <c r="N598" s="5" t="n"/>
-      <c r="P598" s="5" t="n"/>
     </row>
     <row r="599">
       <c r="N599" s="5" t="n"/>
-      <c r="P599" s="5" t="n"/>
     </row>
     <row r="600">
       <c r="N600" s="5" t="n"/>
-      <c r="P600" s="5" t="n"/>
     </row>
     <row r="601">
       <c r="N601" s="5" t="n"/>
-      <c r="P601" s="5" t="n"/>
     </row>
     <row r="602">
       <c r="N602" s="5" t="n"/>
-      <c r="P602" s="5" t="n"/>
     </row>
     <row r="603">
       <c r="N603" s="5" t="n"/>
-      <c r="P603" s="5" t="n"/>
     </row>
     <row r="604">
       <c r="N604" s="5" t="n"/>
-      <c r="P604" s="5" t="n"/>
     </row>
     <row r="605">
       <c r="N605" s="5" t="n"/>
-      <c r="P605" s="5" t="n"/>
     </row>
     <row r="606">
       <c r="N606" s="5" t="n"/>
-      <c r="P606" s="5" t="n"/>
     </row>
     <row r="607">
       <c r="N607" s="5" t="n"/>
-      <c r="P607" s="5" t="n"/>
     </row>
     <row r="608">
       <c r="N608" s="5" t="n"/>
-      <c r="P608" s="5" t="n"/>
     </row>
     <row r="609">
       <c r="N609" s="5" t="n"/>
-      <c r="P609" s="5" t="n"/>
     </row>
     <row r="610">
       <c r="N610" s="5" t="n"/>
-      <c r="P610" s="5" t="n"/>
     </row>
     <row r="611">
       <c r="N611" s="5" t="n"/>
-      <c r="P611" s="5" t="n"/>
     </row>
     <row r="612">
       <c r="N612" s="5" t="n"/>
-      <c r="P612" s="5" t="n"/>
     </row>
     <row r="613">
       <c r="N613" s="5" t="n"/>
-      <c r="P613" s="5" t="n"/>
     </row>
     <row r="614">
       <c r="N614" s="5" t="n"/>
-      <c r="P614" s="5" t="n"/>
     </row>
     <row r="615">
       <c r="N615" s="5" t="n"/>
-      <c r="P615" s="5" t="n"/>
     </row>
     <row r="616">
       <c r="N616" s="5" t="n"/>
-      <c r="P616" s="5" t="n"/>
     </row>
     <row r="617">
       <c r="N617" s="5" t="n"/>
-      <c r="P617" s="5" t="n"/>
     </row>
     <row r="618">
       <c r="N618" s="5" t="n"/>
-      <c r="P618" s="5" t="n"/>
     </row>
     <row r="619">
       <c r="N619" s="5" t="n"/>
-      <c r="P619" s="5" t="n"/>
     </row>
     <row r="620">
       <c r="N620" s="5" t="n"/>
-      <c r="P620" s="5" t="n"/>
     </row>
     <row r="621">
       <c r="N621" s="5" t="n"/>
-      <c r="P621" s="5" t="n"/>
     </row>
     <row r="622">
       <c r="N622" s="5" t="n"/>
-      <c r="P622" s="5" t="n"/>
     </row>
     <row r="623">
       <c r="N623" s="5" t="n"/>
-      <c r="P623" s="5" t="n"/>
     </row>
     <row r="624">
       <c r="N624" s="5" t="n"/>
-      <c r="P624" s="5" t="n"/>
     </row>
     <row r="625">
       <c r="N625" s="5" t="n"/>
-      <c r="P625" s="5" t="n"/>
     </row>
     <row r="626">
       <c r="N626" s="5" t="n"/>
-      <c r="P626" s="5" t="n"/>
     </row>
     <row r="627">
       <c r="N627" s="5" t="n"/>
-      <c r="P627" s="5" t="n"/>
     </row>
     <row r="628">
       <c r="N628" s="5" t="n"/>
-      <c r="P628" s="5" t="n"/>
     </row>
     <row r="629">
       <c r="N629" s="5" t="n"/>
-      <c r="P629" s="5" t="n"/>
     </row>
     <row r="630">
       <c r="N630" s="5" t="n"/>
-      <c r="P630" s="5" t="n"/>
     </row>
     <row r="631">
       <c r="N631" s="5" t="n"/>
-      <c r="P631" s="5" t="n"/>
     </row>
     <row r="632">
       <c r="N632" s="5" t="n"/>
-      <c r="P632" s="5" t="n"/>
     </row>
     <row r="633">
       <c r="N633" s="5" t="n"/>
-      <c r="P633" s="5" t="n"/>
     </row>
     <row r="634">
       <c r="N634" s="5" t="n"/>
-      <c r="P634" s="5" t="n"/>
     </row>
     <row r="635">
       <c r="N635" s="5" t="n"/>
-      <c r="P635" s="5" t="n"/>
     </row>
     <row r="636">
       <c r="N636" s="5" t="n"/>
-      <c r="P636" s="5" t="n"/>
     </row>
     <row r="637">
       <c r="N637" s="5" t="n"/>
-      <c r="P637" s="5" t="n"/>
     </row>
     <row r="638">
       <c r="N638" s="5" t="n"/>
-      <c r="P638" s="5" t="n"/>
     </row>
     <row r="639">
       <c r="N639" s="5" t="n"/>
-      <c r="P639" s="5" t="n"/>
     </row>
     <row r="640">
       <c r="N640" s="5" t="n"/>
-      <c r="P640" s="5" t="n"/>
     </row>
     <row r="641">
       <c r="N641" s="5" t="n"/>
-      <c r="P641" s="5" t="n"/>
     </row>
     <row r="642">
       <c r="N642" s="5" t="n"/>
-      <c r="P642" s="5" t="n"/>
     </row>
     <row r="643">
       <c r="N643" s="5" t="n"/>
-      <c r="P643" s="5" t="n"/>
     </row>
     <row r="644">
       <c r="N644" s="5" t="n"/>
-      <c r="P644" s="5" t="n"/>
     </row>
     <row r="645">
       <c r="N645" s="5" t="n"/>
-      <c r="P645" s="5" t="n"/>
     </row>
     <row r="646">
       <c r="N646" s="5" t="n"/>
-      <c r="P646" s="5" t="n"/>
     </row>
     <row r="647">
       <c r="N647" s="5" t="n"/>
-      <c r="P647" s="5" t="n"/>
     </row>
     <row r="648">
       <c r="N648" s="5" t="n"/>
-      <c r="P648" s="5" t="n"/>
     </row>
     <row r="649">
       <c r="N649" s="5" t="n"/>
-      <c r="P649" s="5" t="n"/>
     </row>
     <row r="650">
       <c r="N650" s="5" t="n"/>
-      <c r="P650" s="5" t="n"/>
     </row>
     <row r="651">
       <c r="N651" s="5" t="n"/>
-      <c r="P651" s="5" t="n"/>
     </row>
     <row r="652">
       <c r="N652" s="5" t="n"/>
-      <c r="P652" s="5" t="n"/>
     </row>
     <row r="653">
       <c r="N653" s="5" t="n"/>
-      <c r="P653" s="5" t="n"/>
     </row>
     <row r="654">
       <c r="N654" s="5" t="n"/>
-      <c r="P654" s="5" t="n"/>
     </row>
     <row r="655">
       <c r="N655" s="5" t="n"/>
-      <c r="P655" s="5" t="n"/>
     </row>
     <row r="656">
       <c r="N656" s="5" t="n"/>
-      <c r="P656" s="5" t="n"/>
     </row>
     <row r="657">
       <c r="N657" s="5" t="n"/>
-      <c r="P657" s="5" t="n"/>
     </row>
     <row r="658">
       <c r="N658" s="5" t="n"/>
-      <c r="P658" s="5" t="n"/>
     </row>
     <row r="659">
       <c r="N659" s="5" t="n"/>
-      <c r="P659" s="5" t="n"/>
     </row>
     <row r="660">
       <c r="N660" s="5" t="n"/>
-      <c r="P660" s="5" t="n"/>
     </row>
     <row r="661">
       <c r="N661" s="5" t="n"/>
-      <c r="P661" s="5" t="n"/>
     </row>
     <row r="662">
       <c r="N662" s="5" t="n"/>
-      <c r="P662" s="5" t="n"/>
     </row>
     <row r="663">
       <c r="N663" s="5" t="n"/>
-      <c r="P663" s="5" t="n"/>
     </row>
     <row r="664">
       <c r="N664" s="5" t="n"/>
-      <c r="P664" s="5" t="n"/>
     </row>
     <row r="665">
       <c r="N665" s="5" t="n"/>
-      <c r="P665" s="5" t="n"/>
     </row>
     <row r="666">
       <c r="N666" s="5" t="n"/>
-      <c r="P666" s="5" t="n"/>
     </row>
     <row r="667">
       <c r="N667" s="5" t="n"/>
-      <c r="P667" s="5" t="n"/>
     </row>
     <row r="668">
       <c r="N668" s="5" t="n"/>
-      <c r="P668" s="5" t="n"/>
     </row>
     <row r="669">
       <c r="N669" s="5" t="n"/>
-      <c r="P669" s="5" t="n"/>
     </row>
     <row r="670">
       <c r="N670" s="5" t="n"/>
-      <c r="P670" s="5" t="n"/>
     </row>
     <row r="671">
       <c r="N671" s="5" t="n"/>
-      <c r="P671" s="5" t="n"/>
     </row>
     <row r="672">
       <c r="N672" s="5" t="n"/>
-      <c r="P672" s="5" t="n"/>
     </row>
     <row r="673">
       <c r="N673" s="5" t="n"/>
-      <c r="P673" s="5" t="n"/>
     </row>
     <row r="674">
       <c r="N674" s="5" t="n"/>
-      <c r="P674" s="5" t="n"/>
     </row>
     <row r="675">
       <c r="N675" s="5" t="n"/>
-      <c r="P675" s="5" t="n"/>
     </row>
     <row r="676">
       <c r="N676" s="5" t="n"/>
-      <c r="P676" s="5" t="n"/>
     </row>
     <row r="677">
       <c r="N677" s="5" t="n"/>
-      <c r="P677" s="5" t="n"/>
     </row>
     <row r="678">
       <c r="N678" s="5" t="n"/>
-      <c r="P678" s="5" t="n"/>
     </row>
     <row r="679">
       <c r="N679" s="5" t="n"/>
-      <c r="P679" s="5" t="n"/>
     </row>
     <row r="680">
       <c r="N680" s="5" t="n"/>
-      <c r="P680" s="5" t="n"/>
     </row>
     <row r="681">
       <c r="N681" s="5" t="n"/>
-      <c r="P681" s="5" t="n"/>
     </row>
     <row r="682">
       <c r="N682" s="5" t="n"/>
-      <c r="P682" s="5" t="n"/>
     </row>
     <row r="683">
       <c r="N683" s="5" t="n"/>
-      <c r="P683" s="5" t="n"/>
     </row>
     <row r="684">
       <c r="N684" s="5" t="n"/>
-      <c r="P684" s="5" t="n"/>
     </row>
     <row r="685">
       <c r="N685" s="5" t="n"/>
-      <c r="P685" s="5" t="n"/>
     </row>
     <row r="686">
       <c r="N686" s="5" t="n"/>
-      <c r="P686" s="5" t="n"/>
     </row>
     <row r="687">
       <c r="N687" s="5" t="n"/>
-      <c r="P687" s="5" t="n"/>
     </row>
     <row r="688">
       <c r="N688" s="5" t="n"/>
-      <c r="P688" s="5" t="n"/>
     </row>
     <row r="689">
       <c r="N689" s="5" t="n"/>
-      <c r="P689" s="5" t="n"/>
     </row>
     <row r="690">
       <c r="N690" s="5" t="n"/>
-      <c r="P690" s="5" t="n"/>
     </row>
     <row r="691">
       <c r="N691" s="5" t="n"/>
-      <c r="P691" s="5" t="n"/>
     </row>
     <row r="692">
       <c r="N692" s="5" t="n"/>
-      <c r="P692" s="5" t="n"/>
     </row>
     <row r="693">
       <c r="N693" s="5" t="n"/>
-      <c r="P693" s="5" t="n"/>
     </row>
     <row r="694">
       <c r="N694" s="5" t="n"/>
-      <c r="P694" s="5" t="n"/>
     </row>
     <row r="695">
       <c r="N695" s="5" t="n"/>
-      <c r="P695" s="5" t="n"/>
     </row>
     <row r="696">
       <c r="N696" s="5" t="n"/>
-      <c r="P696" s="5" t="n"/>
     </row>
     <row r="697">
       <c r="N697" s="5" t="n"/>
-      <c r="P697" s="5" t="n"/>
     </row>
     <row r="698">
       <c r="N698" s="5" t="n"/>
-      <c r="P698" s="5" t="n"/>
     </row>
     <row r="699">
       <c r="N699" s="5" t="n"/>
-      <c r="P699" s="5" t="n"/>
     </row>
     <row r="700">
       <c r="N700" s="5" t="n"/>
-      <c r="P700" s="5" t="n"/>
     </row>
     <row r="701">
       <c r="N701" s="5" t="n"/>
-      <c r="P701" s="5" t="n"/>
     </row>
     <row r="702">
       <c r="N702" s="5" t="n"/>
-      <c r="P702" s="5" t="n"/>
     </row>
     <row r="703">
       <c r="N703" s="5" t="n"/>
-      <c r="P703" s="5" t="n"/>
     </row>
     <row r="704">
       <c r="N704" s="5" t="n"/>
-      <c r="P704" s="5" t="n"/>
     </row>
     <row r="705">
       <c r="N705" s="5" t="n"/>
-      <c r="P705" s="5" t="n"/>
     </row>
     <row r="706">
       <c r="N706" s="5" t="n"/>
-      <c r="P706" s="5" t="n"/>
     </row>
     <row r="707">
       <c r="N707" s="5" t="n"/>
-      <c r="P707" s="5" t="n"/>
     </row>
     <row r="708">
       <c r="N708" s="5" t="n"/>
-      <c r="P708" s="5" t="n"/>
     </row>
     <row r="709">
       <c r="N709" s="5" t="n"/>
-      <c r="P709" s="5" t="n"/>
     </row>
     <row r="710">
       <c r="N710" s="5" t="n"/>
-      <c r="P710" s="5" t="n"/>
     </row>
     <row r="711">
       <c r="N711" s="5" t="n"/>
-      <c r="P711" s="5" t="n"/>
     </row>
     <row r="712">
       <c r="N712" s="5" t="n"/>
-      <c r="P712" s="5" t="n"/>
     </row>
     <row r="713">
       <c r="N713" s="5" t="n"/>
-      <c r="P713" s="5" t="n"/>
     </row>
     <row r="714">
       <c r="N714" s="5" t="n"/>
-      <c r="P714" s="5" t="n"/>
     </row>
     <row r="715">
       <c r="N715" s="5" t="n"/>
-      <c r="P715" s="5" t="n"/>
     </row>
     <row r="716">
       <c r="N716" s="5" t="n"/>
-      <c r="P716" s="5" t="n"/>
     </row>
     <row r="717">
       <c r="N717" s="5" t="n"/>
-      <c r="P717" s="5" t="n"/>
     </row>
     <row r="718">
       <c r="N718" s="5" t="n"/>
-      <c r="P718" s="5" t="n"/>
     </row>
     <row r="719">
       <c r="N719" s="5" t="n"/>
-      <c r="P719" s="5" t="n"/>
     </row>
     <row r="720">
       <c r="N720" s="5" t="n"/>
-      <c r="P720" s="5" t="n"/>
     </row>
     <row r="721">
       <c r="N721" s="5" t="n"/>
-      <c r="P721" s="5" t="n"/>
     </row>
     <row r="722">
       <c r="N722" s="5" t="n"/>
-      <c r="P722" s="5" t="n"/>
     </row>
     <row r="723">
       <c r="N723" s="5" t="n"/>
-      <c r="P723" s="5" t="n"/>
     </row>
     <row r="724">
       <c r="N724" s="5" t="n"/>
-      <c r="P724" s="5" t="n"/>
     </row>
     <row r="725">
       <c r="N725" s="5" t="n"/>
-      <c r="P725" s="5" t="n"/>
     </row>
     <row r="726">
       <c r="N726" s="5" t="n"/>
-      <c r="P726" s="5" t="n"/>
     </row>
     <row r="727">
       <c r="N727" s="5" t="n"/>
-      <c r="P727" s="5" t="n"/>
     </row>
     <row r="728">
       <c r="N728" s="5" t="n"/>
-      <c r="P728" s="5" t="n"/>
     </row>
     <row r="729">
       <c r="N729" s="5" t="n"/>
-      <c r="P729" s="5" t="n"/>
     </row>
     <row r="730">
       <c r="N730" s="5" t="n"/>
-      <c r="P730" s="5" t="n"/>
     </row>
     <row r="731">
       <c r="N731" s="5" t="n"/>
-      <c r="P731" s="5" t="n"/>
     </row>
     <row r="732">
       <c r="N732" s="5" t="n"/>
-      <c r="P732" s="5" t="n"/>
     </row>
     <row r="733">
       <c r="N733" s="5" t="n"/>
-      <c r="P733" s="5" t="n"/>
     </row>
     <row r="734">
       <c r="N734" s="5" t="n"/>
-      <c r="P734" s="5" t="n"/>
     </row>
     <row r="735">
       <c r="N735" s="5" t="n"/>
-      <c r="P735" s="5" t="n"/>
     </row>
     <row r="736">
       <c r="N736" s="5" t="n"/>
-      <c r="P736" s="5" t="n"/>
     </row>
     <row r="737">
       <c r="N737" s="5" t="n"/>
-      <c r="P737" s="5" t="n"/>
     </row>
     <row r="738">
       <c r="N738" s="5" t="n"/>
-      <c r="P738" s="5" t="n"/>
     </row>
     <row r="739">
       <c r="N739" s="5" t="n"/>
-      <c r="P739" s="5" t="n"/>
     </row>
     <row r="740">
       <c r="N740" s="5" t="n"/>
-      <c r="P740" s="5" t="n"/>
     </row>
     <row r="741">
       <c r="N741" s="5" t="n"/>
-      <c r="P741" s="5" t="n"/>
     </row>
     <row r="742">
       <c r="N742" s="5" t="n"/>
-      <c r="P742" s="5" t="n"/>
     </row>
     <row r="743">
       <c r="N743" s="5" t="n"/>
-      <c r="P743" s="5" t="n"/>
     </row>
     <row r="744">
       <c r="N744" s="5" t="n"/>
-      <c r="P744" s="5" t="n"/>
     </row>
     <row r="745">
       <c r="N745" s="5" t="n"/>
-      <c r="P745" s="5" t="n"/>
     </row>
     <row r="746">
       <c r="N746" s="5" t="n"/>
-      <c r="P746" s="5" t="n"/>
     </row>
     <row r="747">
       <c r="N747" s="5" t="n"/>
-      <c r="P747" s="5" t="n"/>
     </row>
     <row r="748">
       <c r="N748" s="5" t="n"/>
-      <c r="P748" s="5" t="n"/>
     </row>
     <row r="749">
       <c r="N749" s="5" t="n"/>
-      <c r="P749" s="5" t="n"/>
     </row>
     <row r="750">
       <c r="N750" s="5" t="n"/>
-      <c r="P750" s="5" t="n"/>
     </row>
     <row r="751">
       <c r="N751" s="5" t="n"/>
-      <c r="P751" s="5" t="n"/>
     </row>
     <row r="752">
       <c r="N752" s="5" t="n"/>
-      <c r="P752" s="5" t="n"/>
     </row>
     <row r="753">
       <c r="N753" s="5" t="n"/>
-      <c r="P753" s="5" t="n"/>
     </row>
     <row r="754">
       <c r="N754" s="5" t="n"/>
-      <c r="P754" s="5" t="n"/>
     </row>
     <row r="755">
       <c r="N755" s="5" t="n"/>
-      <c r="P755" s="5" t="n"/>
     </row>
     <row r="756">
       <c r="N756" s="5" t="n"/>
-      <c r="P756" s="5" t="n"/>
     </row>
     <row r="757">
       <c r="N757" s="5" t="n"/>
-      <c r="P757" s="5" t="n"/>
     </row>
     <row r="758">
       <c r="N758" s="5" t="n"/>
-      <c r="P758" s="5" t="n"/>
     </row>
     <row r="759">
       <c r="N759" s="5" t="n"/>
-      <c r="P759" s="5" t="n"/>
     </row>
     <row r="760">
       <c r="N760" s="5" t="n"/>
-      <c r="P760" s="5" t="n"/>
     </row>
     <row r="761">
       <c r="N761" s="5" t="n"/>
-      <c r="P761" s="5" t="n"/>
     </row>
     <row r="762">
       <c r="N762" s="5" t="n"/>
-      <c r="P762" s="5" t="n"/>
     </row>
     <row r="763">
       <c r="N763" s="5" t="n"/>
-      <c r="P763" s="5" t="n"/>
     </row>
     <row r="764">
       <c r="N764" s="5" t="n"/>
-      <c r="P764" s="5" t="n"/>
     </row>
     <row r="765">
       <c r="N765" s="5" t="n"/>
-      <c r="P765" s="5" t="n"/>
     </row>
     <row r="766">
       <c r="N766" s="5" t="n"/>
-      <c r="P766" s="5" t="n"/>
     </row>
     <row r="767">
       <c r="N767" s="5" t="n"/>
-      <c r="P767" s="5" t="n"/>
     </row>
     <row r="768">
       <c r="N768" s="5" t="n"/>
-      <c r="P768" s="5" t="n"/>
     </row>
     <row r="769">
       <c r="N769" s="5" t="n"/>
-      <c r="P769" s="5" t="n"/>
     </row>
     <row r="770">
       <c r="N770" s="5" t="n"/>
-      <c r="P770" s="5" t="n"/>
     </row>
     <row r="771">
       <c r="N771" s="5" t="n"/>
-      <c r="P771" s="5" t="n"/>
     </row>
     <row r="772">
       <c r="N772" s="5" t="n"/>
-      <c r="P772" s="5" t="n"/>
     </row>
     <row r="773">
       <c r="N773" s="5" t="n"/>
-      <c r="P773" s="5" t="n"/>
     </row>
     <row r="774">
       <c r="N774" s="5" t="n"/>
-      <c r="P774" s="5" t="n"/>
     </row>
     <row r="775">
       <c r="N775" s="5" t="n"/>
-      <c r="P775" s="5" t="n"/>
     </row>
     <row r="776">
       <c r="N776" s="5" t="n"/>
-      <c r="P776" s="5" t="n"/>
     </row>
     <row r="777">
       <c r="N777" s="5" t="n"/>
-      <c r="P777" s="5" t="n"/>
     </row>
     <row r="778">
       <c r="N778" s="5" t="n"/>
-      <c r="P778" s="5" t="n"/>
     </row>
     <row r="779">
       <c r="N779" s="5" t="n"/>
-      <c r="P779" s="5" t="n"/>
     </row>
     <row r="780">
       <c r="N780" s="5" t="n"/>
-      <c r="P780" s="5" t="n"/>
     </row>
     <row r="781">
       <c r="N781" s="5" t="n"/>
-      <c r="P781" s="5" t="n"/>
     </row>
     <row r="782">
       <c r="N782" s="5" t="n"/>
-      <c r="P782" s="5" t="n"/>
     </row>
     <row r="783">
       <c r="N783" s="5" t="n"/>
-      <c r="P783" s="5" t="n"/>
     </row>
     <row r="784">
       <c r="N784" s="5" t="n"/>
-      <c r="P784" s="5" t="n"/>
     </row>
     <row r="785">
       <c r="N785" s="5" t="n"/>
-      <c r="P785" s="5" t="n"/>
     </row>
     <row r="786">
       <c r="N786" s="5" t="n"/>
-      <c r="P786" s="5" t="n"/>
     </row>
     <row r="787">
       <c r="N787" s="5" t="n"/>
-      <c r="P787" s="5" t="n"/>
     </row>
     <row r="788">
       <c r="N788" s="5" t="n"/>
-      <c r="P788" s="5" t="n"/>
     </row>
     <row r="789">
       <c r="N789" s="5" t="n"/>
-      <c r="P789" s="5" t="n"/>
     </row>
     <row r="790">
       <c r="N790" s="5" t="n"/>
-      <c r="P790" s="5" t="n"/>
     </row>
     <row r="791">
       <c r="N791" s="5" t="n"/>
-      <c r="P791" s="5" t="n"/>
     </row>
     <row r="792">
       <c r="N792" s="5" t="n"/>
-      <c r="P792" s="5" t="n"/>
     </row>
     <row r="793">
       <c r="N793" s="5" t="n"/>
-      <c r="P793" s="5" t="n"/>
     </row>
     <row r="794">
       <c r="N794" s="5" t="n"/>
-      <c r="P794" s="5" t="n"/>
     </row>
     <row r="795">
       <c r="N795" s="5" t="n"/>
-      <c r="P795" s="5" t="n"/>
     </row>
     <row r="796">
       <c r="N796" s="5" t="n"/>
-      <c r="P796" s="5" t="n"/>
     </row>
     <row r="797">
       <c r="N797" s="5" t="n"/>
-      <c r="P797" s="5" t="n"/>
     </row>
     <row r="798">
       <c r="N798" s="5" t="n"/>
-      <c r="P798" s="5" t="n"/>
     </row>
     <row r="799">
       <c r="N799" s="5" t="n"/>
-      <c r="P799" s="5" t="n"/>
     </row>
     <row r="800">
       <c r="N800" s="5" t="n"/>
-      <c r="P800" s="5" t="n"/>
     </row>
     <row r="801">
       <c r="N801" s="5" t="n"/>
-      <c r="P801" s="5" t="n"/>
     </row>
     <row r="802">
       <c r="N802" s="5" t="n"/>
-      <c r="P802" s="5" t="n"/>
     </row>
     <row r="803">
       <c r="N803" s="5" t="n"/>
-      <c r="P803" s="5" t="n"/>
     </row>
     <row r="804">
       <c r="N804" s="5" t="n"/>
-      <c r="P804" s="5" t="n"/>
     </row>
     <row r="805">
       <c r="N805" s="5" t="n"/>
-      <c r="P805" s="5" t="n"/>
     </row>
     <row r="806">
       <c r="N806" s="5" t="n"/>
-      <c r="P806" s="5" t="n"/>
     </row>
     <row r="807">
       <c r="N807" s="5" t="n"/>
-      <c r="P807" s="5" t="n"/>
     </row>
     <row r="808">
       <c r="N808" s="5" t="n"/>
-      <c r="P808" s="5" t="n"/>
     </row>
     <row r="809">
       <c r="N809" s="5" t="n"/>
-      <c r="P809" s="5" t="n"/>
     </row>
     <row r="810">
       <c r="N810" s="5" t="n"/>
-      <c r="P810" s="5" t="n"/>
     </row>
     <row r="811">
       <c r="N811" s="5" t="n"/>
-      <c r="P811" s="5" t="n"/>
     </row>
     <row r="812">
       <c r="N812" s="5" t="n"/>
-      <c r="P812" s="5" t="n"/>
     </row>
     <row r="813">
       <c r="N813" s="5" t="n"/>
-      <c r="P813" s="5" t="n"/>
     </row>
     <row r="814">
       <c r="N814" s="5" t="n"/>
-      <c r="P814" s="5" t="n"/>
     </row>
     <row r="815">
       <c r="N815" s="5" t="n"/>
-      <c r="P815" s="5" t="n"/>
     </row>
     <row r="816">
       <c r="N816" s="5" t="n"/>
-      <c r="P816" s="5" t="n"/>
     </row>
     <row r="817">
       <c r="N817" s="5" t="n"/>
-      <c r="P817" s="5" t="n"/>
     </row>
     <row r="818">
       <c r="N818" s="5" t="n"/>
-      <c r="P818" s="5" t="n"/>
     </row>
     <row r="819">
       <c r="N819" s="5" t="n"/>
-      <c r="P819" s="5" t="n"/>
     </row>
     <row r="820">
       <c r="N820" s="5" t="n"/>
-      <c r="P820" s="5" t="n"/>
     </row>
     <row r="821">
       <c r="N821" s="5" t="n"/>
-      <c r="P821" s="5" t="n"/>
     </row>
     <row r="822">
       <c r="N822" s="5" t="n"/>
-      <c r="P822" s="5" t="n"/>
     </row>
     <row r="823">
       <c r="N823" s="5" t="n"/>
-      <c r="P823" s="5" t="n"/>
     </row>
     <row r="824">
       <c r="N824" s="5" t="n"/>
-      <c r="P824" s="5" t="n"/>
     </row>
     <row r="825">
       <c r="N825" s="5" t="n"/>
-      <c r="P825" s="5" t="n"/>
     </row>
     <row r="826">
       <c r="N826" s="5" t="n"/>
-      <c r="P826" s="5" t="n"/>
     </row>
     <row r="827">
       <c r="N827" s="5" t="n"/>
-      <c r="P827" s="5" t="n"/>
     </row>
     <row r="828">
       <c r="N828" s="5" t="n"/>
-      <c r="P828" s="5" t="n"/>
     </row>
     <row r="829">
       <c r="N829" s="5" t="n"/>
-      <c r="P829" s="5" t="n"/>
     </row>
     <row r="830">
       <c r="N830" s="5" t="n"/>
-      <c r="P830" s="5" t="n"/>
     </row>
     <row r="831">
       <c r="N831" s="5" t="n"/>
-      <c r="P831" s="5" t="n"/>
     </row>
     <row r="832">
       <c r="N832" s="5" t="n"/>
-      <c r="P832" s="5" t="n"/>
     </row>
     <row r="833">
       <c r="N833" s="5" t="n"/>
-      <c r="P833" s="5" t="n"/>
     </row>
     <row r="834">
       <c r="N834" s="5" t="n"/>
-      <c r="P834" s="5" t="n"/>
     </row>
     <row r="835">
       <c r="N835" s="5" t="n"/>
-      <c r="P835" s="5" t="n"/>
     </row>
     <row r="836">
       <c r="N836" s="5" t="n"/>
-      <c r="P836" s="5" t="n"/>
     </row>
     <row r="837">
       <c r="N837" s="5" t="n"/>
-      <c r="P837" s="5" t="n"/>
     </row>
     <row r="838">
       <c r="N838" s="5" t="n"/>
-      <c r="P838" s="5" t="n"/>
     </row>
     <row r="839">
       <c r="N839" s="5" t="n"/>
-      <c r="P839" s="5" t="n"/>
     </row>
     <row r="840">
       <c r="N840" s="5" t="n"/>
-      <c r="P840" s="5" t="n"/>
     </row>
     <row r="841">
       <c r="N841" s="5" t="n"/>
-      <c r="P841" s="5" t="n"/>
     </row>
     <row r="842">
       <c r="N842" s="5" t="n"/>
-      <c r="P842" s="5" t="n"/>
     </row>
     <row r="843">
       <c r="N843" s="5" t="n"/>
-      <c r="P843" s="5" t="n"/>
     </row>
     <row r="844">
       <c r="N844" s="5" t="n"/>
-      <c r="P844" s="5" t="n"/>
     </row>
     <row r="845">
       <c r="N845" s="5" t="n"/>
-      <c r="P845" s="5" t="n"/>
     </row>
     <row r="846">
       <c r="N846" s="5" t="n"/>
-      <c r="P846" s="5" t="n"/>
     </row>
     <row r="847">
       <c r="N847" s="5" t="n"/>
-      <c r="P847" s="5" t="n"/>
     </row>
     <row r="848">
       <c r="N848" s="5" t="n"/>
-      <c r="P848" s="5" t="n"/>
     </row>
     <row r="849">
       <c r="N849" s="5" t="n"/>
-      <c r="P849" s="5" t="n"/>
     </row>
     <row r="850">
       <c r="N850" s="5" t="n"/>
-      <c r="P850" s="5" t="n"/>
     </row>
     <row r="851">
       <c r="N851" s="5" t="n"/>
-      <c r="P851" s="5" t="n"/>
     </row>
     <row r="852">
       <c r="N852" s="5" t="n"/>
-      <c r="P852" s="5" t="n"/>
     </row>
     <row r="853">
       <c r="N853" s="5" t="n"/>
-      <c r="P853" s="5" t="n"/>
     </row>
     <row r="854">
       <c r="N854" s="5" t="n"/>
-      <c r="P854" s="5" t="n"/>
     </row>
     <row r="855">
       <c r="N855" s="5" t="n"/>
-      <c r="P855" s="5" t="n"/>
     </row>
     <row r="856">
       <c r="N856" s="5" t="n"/>
-      <c r="P856" s="5" t="n"/>
     </row>
     <row r="857">
       <c r="N857" s="5" t="n"/>
-      <c r="P857" s="5" t="n"/>
     </row>
     <row r="858">
       <c r="N858" s="5" t="n"/>
-      <c r="P858" s="5" t="n"/>
     </row>
     <row r="859">
       <c r="N859" s="5" t="n"/>
-      <c r="P859" s="5" t="n"/>
     </row>
     <row r="860">
       <c r="N860" s="5" t="n"/>
-      <c r="P860" s="5" t="n"/>
     </row>
     <row r="861">
       <c r="N861" s="5" t="n"/>
-      <c r="P861" s="5" t="n"/>
     </row>
     <row r="862">
       <c r="N862" s="5" t="n"/>
-      <c r="P862" s="5" t="n"/>
     </row>
     <row r="863">
       <c r="N863" s="5" t="n"/>
-      <c r="P863" s="5" t="n"/>
     </row>
     <row r="864">
       <c r="N864" s="5" t="n"/>
-      <c r="P864" s="5" t="n"/>
     </row>
     <row r="865">
       <c r="N865" s="5" t="n"/>
-      <c r="P865" s="5" t="n"/>
     </row>
     <row r="866">
       <c r="N866" s="5" t="n"/>
-      <c r="P866" s="5" t="n"/>
     </row>
     <row r="867">
       <c r="N867" s="5" t="n"/>
-      <c r="P867" s="5" t="n"/>
     </row>
     <row r="868">
       <c r="N868" s="5" t="n"/>
-      <c r="P868" s="5" t="n"/>
     </row>
     <row r="869">
       <c r="N869" s="5" t="n"/>
-      <c r="P869" s="5" t="n"/>
     </row>
     <row r="870">
       <c r="N870" s="5" t="n"/>
-      <c r="P870" s="5" t="n"/>
     </row>
     <row r="871">
       <c r="N871" s="5" t="n"/>
-      <c r="P871" s="5" t="n"/>
     </row>
     <row r="872">
       <c r="N872" s="5" t="n"/>
-      <c r="P872" s="5" t="n"/>
     </row>
     <row r="873">
       <c r="N873" s="5" t="n"/>
-      <c r="P873" s="5" t="n"/>
     </row>
     <row r="874">
       <c r="N874" s="5" t="n"/>
-      <c r="P874" s="5" t="n"/>
     </row>
     <row r="875">
       <c r="N875" s="5" t="n"/>
-      <c r="P875" s="5" t="n"/>
     </row>
     <row r="876">
       <c r="N876" s="5" t="n"/>
-      <c r="P876" s="5" t="n"/>
     </row>
     <row r="877">
       <c r="N877" s="5" t="n"/>
-      <c r="P877" s="5" t="n"/>
     </row>
     <row r="878">
       <c r="N878" s="5" t="n"/>
-      <c r="P878" s="5" t="n"/>
     </row>
     <row r="879">
       <c r="N879" s="5" t="n"/>
-      <c r="P879" s="5" t="n"/>
     </row>
     <row r="880">
       <c r="N880" s="5" t="n"/>
-      <c r="P880" s="5" t="n"/>
     </row>
     <row r="881">
       <c r="N881" s="5" t="n"/>
-      <c r="P881" s="5" t="n"/>
     </row>
     <row r="882">
       <c r="N882" s="5" t="n"/>
-      <c r="P882" s="5" t="n"/>
     </row>
     <row r="883">
       <c r="N883" s="5" t="n"/>
-      <c r="P883" s="5" t="n"/>
     </row>
     <row r="884">
       <c r="N884" s="5" t="n"/>
-      <c r="P884" s="5" t="n"/>
     </row>
     <row r="885">
       <c r="N885" s="5" t="n"/>
-      <c r="P885" s="5" t="n"/>
     </row>
     <row r="886">
       <c r="N886" s="5" t="n"/>
-      <c r="P886" s="5" t="n"/>
     </row>
     <row r="887">
       <c r="N887" s="5" t="n"/>
-      <c r="P887" s="5" t="n"/>
     </row>
     <row r="888">
       <c r="N888" s="5" t="n"/>
-      <c r="P888" s="5" t="n"/>
     </row>
     <row r="889">
       <c r="N889" s="5" t="n"/>
-      <c r="P889" s="5" t="n"/>
     </row>
     <row r="890">
       <c r="N890" s="5" t="n"/>
-      <c r="P890" s="5" t="n"/>
     </row>
     <row r="891">
       <c r="N891" s="5" t="n"/>
-      <c r="P891" s="5" t="n"/>
     </row>
     <row r="892">
       <c r="N892" s="5" t="n"/>
-      <c r="P892" s="5" t="n"/>
     </row>
     <row r="893">
       <c r="N893" s="5" t="n"/>
-      <c r="P893" s="5" t="n"/>
     </row>
     <row r="894">
       <c r="N894" s="5" t="n"/>
-      <c r="P894" s="5" t="n"/>
     </row>
     <row r="895">
       <c r="N895" s="5" t="n"/>
-      <c r="P895" s="5" t="n"/>
     </row>
     <row r="896">
       <c r="N896" s="5" t="n"/>
-      <c r="P896" s="5" t="n"/>
     </row>
     <row r="897">
       <c r="N897" s="5" t="n"/>
-      <c r="P897" s="5" t="n"/>
     </row>
     <row r="898">
       <c r="N898" s="5" t="n"/>
-      <c r="P898" s="5" t="n"/>
     </row>
     <row r="899">
       <c r="N899" s="5" t="n"/>
-      <c r="P899" s="5" t="n"/>
     </row>
     <row r="900">
       <c r="N900" s="5" t="n"/>
-      <c r="P900" s="5" t="n"/>
     </row>
     <row r="901">
       <c r="N901" s="5" t="n"/>
-      <c r="P901" s="5" t="n"/>
     </row>
     <row r="902">
       <c r="N902" s="5" t="n"/>
-      <c r="P902" s="5" t="n"/>
     </row>
     <row r="903">
       <c r="N903" s="5" t="n"/>
-      <c r="P903" s="5" t="n"/>
     </row>
     <row r="904">
       <c r="N904" s="5" t="n"/>
-      <c r="P904" s="5" t="n"/>
     </row>
     <row r="905">
       <c r="N905" s="5" t="n"/>
-      <c r="P905" s="5" t="n"/>
     </row>
     <row r="906">
       <c r="N906" s="5" t="n"/>
-      <c r="P906" s="5" t="n"/>
     </row>
     <row r="907">
       <c r="N907" s="5" t="n"/>
-      <c r="P907" s="5" t="n"/>
     </row>
     <row r="908">
       <c r="N908" s="5" t="n"/>
-      <c r="P908" s="5" t="n"/>
     </row>
     <row r="909">
       <c r="N909" s="5" t="n"/>
-      <c r="P909" s="5" t="n"/>
     </row>
     <row r="910">
       <c r="N910" s="5" t="n"/>
-      <c r="P910" s="5" t="n"/>
     </row>
     <row r="911">
       <c r="N911" s="5" t="n"/>
-      <c r="P911" s="5" t="n"/>
     </row>
     <row r="912">
       <c r="N912" s="5" t="n"/>
-      <c r="P912" s="5" t="n"/>
     </row>
     <row r="913">
       <c r="N913" s="5" t="n"/>
-      <c r="P913" s="5" t="n"/>
     </row>
     <row r="914">
       <c r="N914" s="5" t="n"/>
-      <c r="P914" s="5" t="n"/>
     </row>
     <row r="915">
       <c r="N915" s="5" t="n"/>
-      <c r="P915" s="5" t="n"/>
     </row>
     <row r="916">
       <c r="N916" s="5" t="n"/>
-      <c r="P916" s="5" t="n"/>
     </row>
     <row r="917">
       <c r="N917" s="5" t="n"/>
-      <c r="P917" s="5" t="n"/>
     </row>
     <row r="918">
       <c r="N918" s="5" t="n"/>
-      <c r="P918" s="5" t="n"/>
     </row>
     <row r="919">
       <c r="N919" s="5" t="n"/>
-      <c r="P919" s="5" t="n"/>
     </row>
     <row r="920">
       <c r="N920" s="5" t="n"/>
-      <c r="P920" s="5" t="n"/>
     </row>
     <row r="921">
       <c r="N921" s="5" t="n"/>
-      <c r="P921" s="5" t="n"/>
     </row>
     <row r="922">
       <c r="N922" s="5" t="n"/>
-      <c r="P922" s="5" t="n"/>
     </row>
     <row r="923">
       <c r="N923" s="5" t="n"/>
-      <c r="P923" s="5" t="n"/>
     </row>
     <row r="924">
       <c r="N924" s="5" t="n"/>
-      <c r="P924" s="5" t="n"/>
     </row>
     <row r="925">
       <c r="N925" s="5" t="n"/>
-      <c r="P925" s="5" t="n"/>
     </row>
     <row r="926">
       <c r="N926" s="5" t="n"/>
-      <c r="P926" s="5" t="n"/>
     </row>
     <row r="927">
       <c r="N927" s="5" t="n"/>
-      <c r="P927" s="5" t="n"/>
     </row>
     <row r="928">
       <c r="N928" s="5" t="n"/>
-      <c r="P928" s="5" t="n"/>
     </row>
     <row r="929">
       <c r="N929" s="5" t="n"/>
-      <c r="P929" s="5" t="n"/>
     </row>
     <row r="930">
       <c r="N930" s="5" t="n"/>
-      <c r="P930" s="5" t="n"/>
     </row>
     <row r="931">
       <c r="N931" s="5" t="n"/>
-      <c r="P931" s="5" t="n"/>
     </row>
     <row r="932">
       <c r="N932" s="5" t="n"/>
-      <c r="P932" s="5" t="n"/>
     </row>
     <row r="933">
       <c r="N933" s="5" t="n"/>
-      <c r="P933" s="5" t="n"/>
     </row>
     <row r="934">
       <c r="N934" s="5" t="n"/>
-      <c r="P934" s="5" t="n"/>
     </row>
     <row r="935">
       <c r="N935" s="5" t="n"/>
-      <c r="P935" s="5" t="n"/>
     </row>
     <row r="936">
       <c r="N936" s="5" t="n"/>
-      <c r="P936" s="5" t="n"/>
     </row>
     <row r="937">
       <c r="N937" s="5" t="n"/>
-      <c r="P937" s="5" t="n"/>
     </row>
     <row r="938">
       <c r="N938" s="5" t="n"/>
-      <c r="P938" s="5" t="n"/>
     </row>
     <row r="939">
       <c r="N939" s="5" t="n"/>
-      <c r="P939" s="5" t="n"/>
     </row>
     <row r="940">
       <c r="N940" s="5" t="n"/>
-      <c r="P940" s="5" t="n"/>
     </row>
     <row r="941">
       <c r="N941" s="5" t="n"/>
-      <c r="P941" s="5" t="n"/>
     </row>
     <row r="942">
       <c r="N942" s="5" t="n"/>
-      <c r="P942" s="5" t="n"/>
     </row>
     <row r="943">
       <c r="N943" s="5" t="n"/>
-      <c r="P943" s="5" t="n"/>
     </row>
     <row r="944">
       <c r="N944" s="5" t="n"/>
-      <c r="P944" s="5" t="n"/>
     </row>
     <row r="945">
       <c r="N945" s="5" t="n"/>
-      <c r="P945" s="5" t="n"/>
     </row>
     <row r="946">
       <c r="N946" s="5" t="n"/>
-      <c r="P946" s="5" t="n"/>
     </row>
     <row r="947">
       <c r="N947" s="5" t="n"/>
-      <c r="P947" s="5" t="n"/>
     </row>
     <row r="948">
       <c r="N948" s="5" t="n"/>
-      <c r="P948" s="5" t="n"/>
     </row>
     <row r="949">
       <c r="N949" s="5" t="n"/>
-      <c r="P949" s="5" t="n"/>
     </row>
     <row r="950">
       <c r="N950" s="5" t="n"/>
-      <c r="P950" s="5" t="n"/>
     </row>
     <row r="951">
       <c r="N951" s="5" t="n"/>
-      <c r="P951" s="5" t="n"/>
     </row>
     <row r="952">
       <c r="N952" s="5" t="n"/>
-      <c r="P952" s="5" t="n"/>
     </row>
     <row r="953">
       <c r="N953" s="5" t="n"/>
-      <c r="P953" s="5" t="n"/>
     </row>
     <row r="954">
       <c r="N954" s="5" t="n"/>
-      <c r="P954" s="5" t="n"/>
     </row>
     <row r="955">
       <c r="N955" s="5" t="n"/>
-      <c r="P955" s="5" t="n"/>
     </row>
     <row r="956">
       <c r="N956" s="5" t="n"/>
-      <c r="P956" s="5" t="n"/>
     </row>
     <row r="957">
       <c r="N957" s="5" t="n"/>
-      <c r="P957" s="5" t="n"/>
     </row>
     <row r="958">
       <c r="N958" s="5" t="n"/>
-      <c r="P958" s="5" t="n"/>
     </row>
     <row r="959">
       <c r="N959" s="5" t="n"/>
-      <c r="P959" s="5" t="n"/>
     </row>
     <row r="960">
       <c r="N960" s="5" t="n"/>
-      <c r="P960" s="5" t="n"/>
     </row>
     <row r="961">
       <c r="N961" s="5" t="n"/>
-      <c r="P961" s="5" t="n"/>
     </row>
     <row r="962">
       <c r="N962" s="5" t="n"/>
-      <c r="P962" s="5" t="n"/>
     </row>
     <row r="963">
       <c r="N963" s="5" t="n"/>
-      <c r="P963" s="5" t="n"/>
     </row>
     <row r="964">
       <c r="N964" s="5" t="n"/>
-      <c r="P964" s="5" t="n"/>
     </row>
     <row r="965">
       <c r="N965" s="5" t="n"/>
-      <c r="P965" s="5" t="n"/>
     </row>
     <row r="966">
       <c r="N966" s="5" t="n"/>
-      <c r="P966" s="5" t="n"/>
     </row>
     <row r="967">
       <c r="N967" s="5" t="n"/>
-      <c r="P967" s="5" t="n"/>
     </row>
     <row r="968">
       <c r="N968" s="5" t="n"/>
-      <c r="P968" s="5" t="n"/>
     </row>
     <row r="969">
       <c r="N969" s="5" t="n"/>
-      <c r="P969" s="5" t="n"/>
     </row>
     <row r="970">
       <c r="N970" s="5" t="n"/>
-      <c r="P970" s="5" t="n"/>
     </row>
     <row r="971">
       <c r="N971" s="5" t="n"/>
-      <c r="P971" s="5" t="n"/>
     </row>
     <row r="972">
       <c r="N972" s="5" t="n"/>
-      <c r="P972" s="5" t="n"/>
     </row>
     <row r="973">
       <c r="N973" s="5" t="n"/>
-      <c r="P973" s="5" t="n"/>
     </row>
     <row r="974">
       <c r="N974" s="5" t="n"/>
-      <c r="P974" s="5" t="n"/>
     </row>
     <row r="975">
       <c r="N975" s="5" t="n"/>
-      <c r="P975" s="5" t="n"/>
     </row>
     <row r="976">
       <c r="N976" s="5" t="n"/>
-      <c r="P976" s="5" t="n"/>
     </row>
     <row r="977">
       <c r="N977" s="5" t="n"/>
-      <c r="P977" s="5" t="n"/>
     </row>
     <row r="978">
       <c r="N978" s="5" t="n"/>
-      <c r="P978" s="5" t="n"/>
     </row>
     <row r="979">
       <c r="N979" s="5" t="n"/>
-      <c r="P979" s="5" t="n"/>
     </row>
     <row r="980">
       <c r="N980" s="5" t="n"/>
-      <c r="P980" s="5" t="n"/>
     </row>
     <row r="981">
       <c r="N981" s="5" t="n"/>
-      <c r="P981" s="5" t="n"/>
     </row>
     <row r="982">
       <c r="N982" s="5" t="n"/>
-      <c r="P982" s="5" t="n"/>
     </row>
     <row r="983">
       <c r="N983" s="5" t="n"/>
-      <c r="P983" s="5" t="n"/>
     </row>
     <row r="984">
       <c r="N984" s="5" t="n"/>
-      <c r="P984" s="5" t="n"/>
     </row>
     <row r="985">
       <c r="N985" s="5" t="n"/>
-      <c r="P985" s="5" t="n"/>
     </row>
     <row r="986">
       <c r="N986" s="5" t="n"/>
-      <c r="P986" s="5" t="n"/>
     </row>
     <row r="987">
       <c r="N987" s="5" t="n"/>
-      <c r="P987" s="5" t="n"/>
     </row>
     <row r="988">
       <c r="N988" s="5" t="n"/>
-      <c r="P988" s="5" t="n"/>
     </row>
     <row r="989">
       <c r="N989" s="5" t="n"/>
-      <c r="P989" s="5" t="n"/>
     </row>
     <row r="990">
       <c r="N990" s="5" t="n"/>
-      <c r="P990" s="5" t="n"/>
     </row>
     <row r="991">
       <c r="N991" s="5" t="n"/>
-      <c r="P991" s="5" t="n"/>
     </row>
     <row r="992">
       <c r="N992" s="5" t="n"/>
-      <c r="P992" s="5" t="n"/>
     </row>
     <row r="993">
       <c r="N993" s="5" t="n"/>
-      <c r="P993" s="5" t="n"/>
     </row>
     <row r="994">
       <c r="N994" s="5" t="n"/>
-      <c r="P994" s="5" t="n"/>
     </row>
     <row r="995">
       <c r="N995" s="5" t="n"/>
-      <c r="P995" s="5" t="n"/>
     </row>
     <row r="996">
       <c r="N996" s="5" t="n"/>
-      <c r="P996" s="5" t="n"/>
     </row>
     <row r="997">
       <c r="N997" s="5" t="n"/>
-      <c r="P997" s="5" t="n"/>
     </row>
     <row r="998">
       <c r="N998" s="5" t="n"/>
-      <c r="P998" s="5" t="n"/>
     </row>
     <row r="999">
       <c r="N999" s="5" t="n"/>
-      <c r="P999" s="5" t="n"/>
     </row>
     <row r="1000">
       <c r="N1000" s="5" t="n"/>
-      <c r="P1000" s="5" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -4669,7 +3662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B63"/>
+  <dimension ref="B2:B62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="2" max="2"/>
@@ -4740,7 +3733,7 @@
     <row r="12">
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>• Headers: en la FILA 1, columnas A-P (16 columnas).</t>
+          <t>• Headers: en la FILA 1, columnas A-O (15 columnas).</t>
         </is>
       </c>
     </row>
@@ -4771,7 +3764,7 @@
     <row r="17">
       <c r="B17" s="8" t="inlineStr">
         <is>
-          <t>COLUMNAS (16 campos)</t>
+          <t>COLUMNAS (15 campos)</t>
         </is>
       </c>
     </row>
@@ -4785,14 +3778,14 @@
     <row r="19">
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>B  Folio (Manual)           → número o texto. Tu folio interno.</t>
+          <t>B  Folio (Manual)           → folio interno del sistema antiguo.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>C  EXPEDIENTE               → texto libre. Puede quedar vacío.</t>
+          <t>C  EXPEDIENTE               → N° siniestro/expediente del cliente.</t>
         </is>
       </c>
     </row>
@@ -4869,7 +3862,7 @@
     <row r="31">
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>N  Subtotal                 → entero CLP sin separadores. Ej: 30000</t>
+          <t>N  Total                    → entero CLP del servicio. Ej: 30000</t>
         </is>
       </c>
     </row>
@@ -4881,197 +3874,190 @@
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>P  Total                    → entero CLP (con IVA). Ej: 35700</t>
-        </is>
-      </c>
+      <c r="B33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="B34" s="7" t="inlineStr"/>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>NOTA SOBRE EL FORMATO LEGACY ORIGINAL</t>
+        </is>
+      </c>
     </row>
     <row r="35">
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>NOTA SOBRE EL FORMATO LEGACY ORIGINAL</t>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Si subes el archivo "ReporteMemoriasDescriptivas" crudo de la plataforma</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Si subes el archivo "ReporteMemoriasDescriptivas" crudo de la plataforma</t>
+          <t>anterior, el sistema lo acepta también. Las columnas "Ajustador",</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>anterior (con sus 18 columnas originales), el sistema lo acepta también.</t>
+          <t>"Referencia" y "Total" (con IVA) del formato legacy se omiten</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Las columnas "Ajustador" y "Referencia" del formato legacy se omiten</t>
+          <t>automáticamente porque no son relevantes para el análisis.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>automáticamente porque no son relevantes para el análisis.</t>
-        </is>
-      </c>
+      <c r="B39" s="7" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="B40" s="7" t="inlineStr"/>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>FECHAS</t>
+        </is>
+      </c>
     </row>
     <row r="41">
-      <c r="B41" s="8" t="inlineStr">
-        <is>
-          <t>FECHAS</t>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Formato exacto: "DD/MM/AAAA HH:MM:SS a. m." o "DD/MM/AAAA HH:MM:SS p. m."</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Formato exacto: "DD/MM/AAAA HH:MM:SS a. m." o "DD/MM/AAAA HH:MM:SS p. m."</t>
+          <t>Ejemplos válidos:</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Ejemplos válidos:</t>
+          <t xml:space="preserve">   01/09/2020 12:08:00 p. m.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">   01/09/2020 12:08:00 p. m.</t>
+          <t xml:space="preserve">   03/09/2020 10:00:00 a. m.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">   03/09/2020 10:00:00 a. m.</t>
+          <t>Filas con fecha no parseable serán marcadas en el preview y omitidas.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="7" t="inlineStr">
-        <is>
-          <t>Filas con fecha no parseable serán marcadas en el preview y omitidas.</t>
-        </is>
-      </c>
+      <c r="B46" s="7" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="B47" s="7" t="inlineStr"/>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>MONTOS</t>
+        </is>
+      </c>
     </row>
     <row r="48">
-      <c r="B48" s="8" t="inlineStr">
-        <is>
-          <t>MONTOS</t>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>Solo dígitos, sin separadores de miles, sin signo $, sin decimales.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Solo dígitos, sin separadores de miles, sin signo $, sin decimales.</t>
+          <t>✓ Correcto:    30000</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>✓ Correcto:    30000</t>
+          <t>✗ Incorrecto:  $30.000  /  30,000.00  /  30.000</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>✗ Incorrecto:  $30.000  /  30,000.00  /  30.000</t>
-        </is>
-      </c>
+      <c r="B51" s="7" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="B52" s="7" t="inlineStr"/>
+      <c r="B52" s="8" t="inlineStr">
+        <is>
+          <t>PASOS PARA CARGAR</t>
+        </is>
+      </c>
     </row>
     <row r="53">
-      <c r="B53" s="8" t="inlineStr">
-        <is>
-          <t>PASOS PARA CARGAR</t>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>1. Borra la fila ejemplo amarilla (fila 2) — opcional.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>1. Borra la fila ejemplo amarilla (fila 2) — opcional.</t>
+          <t>2. Verifica que no hay filas vacías entre tus datos.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>2. Verifica que no hay filas vacías entre tus datos.</t>
+          <t>3. Guarda como .xlsx (no .xls, no .csv, no Google Sheets).</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>3. Guarda como .xlsx (no .xls, no .csv, no Google Sheets).</t>
+          <t>4. Histórico → tab "Servicios Legacy" → "Importar XLSX".</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>4. Histórico → tab "Servicios Legacy" → "Importar XLSX".</t>
+          <t>5. Revisa el preview antes de confirmar.</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="B58" s="7" t="inlineStr">
-        <is>
-          <t>5. Revisa el preview antes de confirmar.</t>
-        </is>
-      </c>
+      <c r="B58" s="7" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="B59" s="7" t="inlineStr"/>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>CAMPOS LIBRES vs CONTROLADOS</t>
+        </is>
+      </c>
     </row>
     <row r="60">
-      <c r="B60" s="8" t="inlineStr">
-        <is>
-          <t>CAMPOS LIBRES vs CONTROLADOS</t>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>Solo Tipo de servicio (E) y Tipo de vehículo (G) tienen lista cerrada.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>Solo Tipo de servicio (E) y Tipo de vehículo (G) tienen lista cerrada.</t>
+          <t>Aseguradora, Operador y Grúa son texto libre — escríbelos como vengan</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="B62" s="7" t="inlineStr">
-        <is>
-          <t>Aseguradora, Operador y Grúa son texto libre — escríbelos como vengan</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="B63" s="7" t="inlineStr">
         <is>
           <t>en tus respaldos originales. El sistema los acepta tal cual.</t>
         </is>

</xml_diff>